<commit_message>
BGDP AEO 2025 update
</commit_message>
<xml_diff>
--- a/InputData/io-model/BGDP/BAU GDP.xlsx
+++ b/InputData/io-model/BGDP/BAU GDP.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\io-model\BGDP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\io-model\BGDP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E6789F-0E32-4A7C-9717-020DFF41C5DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1FEE6C-D06D-439B-8335-80DF61ADB4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23370" yWindow="465" windowWidth="21600" windowHeight="12735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BEA Data" sheetId="3" r:id="rId2"/>
-    <sheet name="AEO Table 20" sheetId="4" r:id="rId3"/>
-    <sheet name="BGDP" sheetId="2" r:id="rId4"/>
+    <sheet name="AEO 2023 Table 20" sheetId="4" r:id="rId3"/>
+    <sheet name="AEO 2025 Table 20" sheetId="5" r:id="rId4"/>
+    <sheet name="BGDP" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="274">
   <si>
     <t>BGDP BAU Gross Domestic Product</t>
   </si>
@@ -444,6 +445,423 @@
   </si>
   <si>
     <t>2022 to 2012 USD</t>
+  </si>
+  <si>
+    <t>millions</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.KEI_SAL_TRN_LDV_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Unit Sales of Light-Duty Vehicles: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Unit Sales of Light-Duty Vehicles (millions)</t>
+  </si>
+  <si>
+    <t>billion sq ft</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_FLR_COMM_NA_NA_NA_NA_BLNSQFT.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Commercial Floorspace: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Commercial Floorspace (billion square feet)</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_HST_NA_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Housing Starts: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Housing Starts (millions)</t>
+  </si>
+  <si>
+    <t>billion 2012  $</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_PEI_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Real Disposable Personal Income: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Disposable Personal Income</t>
+  </si>
+  <si>
+    <t>percent</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_UER_NA_NA_NA_NA_NA_PCT.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Unemployment Rate: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Unemployment Rate (percentage)</t>
+  </si>
+  <si>
+    <t>2012=1.00</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_LP_NOFM_NA_NA_NA_NA_Y09EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Nonfarm Labor Productivity: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Nonfarm Labor Productivity (2012=1.00)</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_LBF_NA_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Labor Force: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Labor Force (millions)</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.DMG_EMPM_MANF_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Employment, Manufacturing: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Manufacturing</t>
+  </si>
+  <si>
+    <t>Employment</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.DMG_EMPM_NOFM_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Employment, Nonfarm: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nonfarm</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.DMG_POP_65+_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, aged 65 and over: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> aged 65 and over</t>
+  </si>
+  <si>
+    <t>Population</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.DMG_POP_16+_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, aged 16 and over: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> aged 16 and over</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.DMG_POP_PWAF_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, with Armed Forces Overseas: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> with Armed Forces Overseas</t>
+  </si>
+  <si>
+    <t>billion 2012 $</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Total: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_NEINT_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Non-Energy-Intensive: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Non-Energy-Intensive</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_EINT_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Energy-Intensive: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Energy-Intensive</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_MANF_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Manufacturing: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_NMFG_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Agriculture, Mining, and Construction: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> and Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mining</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_IDAL_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Total Industrial: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Total Industrial</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_VOS_NIND_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Non-Industrial: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Non-Industrial and Service Sectors</t>
+  </si>
+  <si>
+    <t>percent, nominal</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_AAUTR_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: AA Utility Bond Rate: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>AA Utility Bond Rate</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_TNR10_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: 10-Year Treasury Note: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>10-Year Treasury Note</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_FFR_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: Federal Funds Rate: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Federal Funds Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> nominal)</t>
+  </si>
+  <si>
+    <t>Interest Rates (percentage</t>
+  </si>
+  <si>
+    <t>1982=1.00</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_WHP_INDCOM_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Industrial Commodities Excluding Energy: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Industrial Commodities excluding Energy</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_WHP_MET_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Metals and Metal Products: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Metals and Metal Products</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_WHP_FULP_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Fuel and Power: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Fuel and Power</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_WHP_NA_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: All Commodities: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>All Commodities</t>
+  </si>
+  <si>
+    <t>Wholesale Price Index (1982=1.00)</t>
+  </si>
+  <si>
+    <t>1982-84=1.00</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_CPI_ENE_NA_IDX82TO84EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Consumer Price Index: Energy Commodities and Services: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Energy Commodities and Services</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_CPI_URB_NA_IDX82TO84EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Consumer Price Index: All-Urban: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>All-urban</t>
+  </si>
+  <si>
+    <t>Consumer Price Index (1982-84=1.00)</t>
+  </si>
+  <si>
+    <t>2012=1.000</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_INDX_NA_NA_GDP_NA_NA_Y09EQ1D3Z.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Price Indices: GDP Chain-type Price Index: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>GDP Chain-type Price Index (2012=1.000)</t>
+  </si>
+  <si>
+    <t>thousand Btu/$ GDP</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.INY_NA_NA_NA_TEN_NA_NA_THBTUPDLRGDP.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Energy Intensity: Total Energy: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Total Energy</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.INY_NA_NA_NA_DELE_NA_NA_THBTUPDLRGDP.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Energy Intensity: Delivered Energy: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Delivered Energy</t>
+  </si>
+  <si>
+    <t>(thousand Btu per 2012 dollar of GDP)</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_RIMP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Imports: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Imports</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_REXP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Exports: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Exports</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_RGSP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Government Spending: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Government Spending</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_RINV_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Business Fixed Investment: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Business Fixed Investment</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_RCNSP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Consumption: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Real Consumption</t>
+  </si>
+  <si>
+    <t>AEO.2025.HIGHZTC.ECI_NA_NA_NA_GDP_REAL_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Real Gross Domestic Product: High Zero-Carbon Technology Cost</t>
+  </si>
+  <si>
+    <t>Growth (2024-2050)</t>
+  </si>
+  <si>
+    <t>units</t>
+  </si>
+  <si>
+    <t>api key</t>
+  </si>
+  <si>
+    <t>full name</t>
+  </si>
+  <si>
+    <t>Source: U.S. Energy Information Administration</t>
+  </si>
+  <si>
+    <t>Tue Dec 02 2025 13:21:36 GMT-0800 (Pacific Standard Time)</t>
+  </si>
+  <si>
+    <t>https://www.eia.gov/outlooks/aeo/data/browser/#/?id=18-AEO2025&amp;cases=highZTC&amp;sourcekey=0</t>
+  </si>
+  <si>
+    <t>Table 20.  Macroeconomic Indicators</t>
+  </si>
+  <si>
+    <t>Annual Energy Outlook 2023 &amp; Annual Energy Outlook 2025</t>
+  </si>
+  <si>
+    <t>High Zero-Carbon Technology Cost Scenario</t>
   </si>
 </sst>
 </file>
@@ -455,7 +873,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -545,8 +963,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -562,6 +987,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -611,7 +1042,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="9">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -631,8 +1062,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -717,8 +1149,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="9" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="9">
+  <cellStyles count="10">
     <cellStyle name="Body: normal cell" xfId="7" xr:uid="{F8888DF3-4DCB-40C2-8840-ADA25445C73F}"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="2" xr:uid="{B8559DFD-85FA-41CB-92D8-B51922D2C5DE}"/>
     <cellStyle name="Footnotes: top row" xfId="8" xr:uid="{20F20C3F-8D2E-4DD4-8407-9E21B5AD66A0}"/>
@@ -727,6 +1165,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="4" xr:uid="{7DAF6620-48AC-4C82-ADAE-1A1B2DCD13C6}"/>
     <cellStyle name="Parent row" xfId="6" xr:uid="{E0037267-FEA4-4DC9-AEE8-91C5C339816D}"/>
+    <cellStyle name="Percent" xfId="9" builtinId="5"/>
     <cellStyle name="Table title" xfId="5" xr:uid="{7CF177E1-AE62-40E6-905A-A3824569EFEA}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1066,7 +1505,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>7</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1077,6 +1516,11 @@
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="34" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9589,6 +10033,15 @@
     <row r="2841" spans="2:32" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B2598:AF2598"/>
+    <mergeCell ref="B2719:AF2719"/>
+    <mergeCell ref="B2837:AF2837"/>
+    <mergeCell ref="B1945:AF1945"/>
+    <mergeCell ref="B2031:AF2031"/>
+    <mergeCell ref="B2153:AF2153"/>
+    <mergeCell ref="B2317:AF2317"/>
+    <mergeCell ref="B2419:AF2419"/>
+    <mergeCell ref="B2509:AF2509"/>
     <mergeCell ref="B1699:AF1699"/>
     <mergeCell ref="B112:AF112"/>
     <mergeCell ref="B308:AF308"/>
@@ -9601,33 +10054,3859 @@
     <mergeCell ref="B1390:AF1390"/>
     <mergeCell ref="B1502:AF1502"/>
     <mergeCell ref="B1604:AF1604"/>
-    <mergeCell ref="B2598:AF2598"/>
-    <mergeCell ref="B2719:AF2719"/>
-    <mergeCell ref="B2837:AF2837"/>
-    <mergeCell ref="B1945:AF1945"/>
-    <mergeCell ref="B2031:AF2031"/>
-    <mergeCell ref="B2153:AF2153"/>
-    <mergeCell ref="B2317:AF2317"/>
-    <mergeCell ref="B2419:AF2419"/>
-    <mergeCell ref="B2509:AF2509"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35A21D9B-71D9-43A1-B63A-6FF08BC567EF}">
+  <dimension ref="A1:AI53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>267</v>
+      </c>
+      <c r="C5" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" t="s">
+        <v>265</v>
+      </c>
+      <c r="E5">
+        <v>2023</v>
+      </c>
+      <c r="F5">
+        <v>2024</v>
+      </c>
+      <c r="G5">
+        <v>2025</v>
+      </c>
+      <c r="H5">
+        <v>2026</v>
+      </c>
+      <c r="I5">
+        <v>2027</v>
+      </c>
+      <c r="J5">
+        <v>2028</v>
+      </c>
+      <c r="K5">
+        <v>2029</v>
+      </c>
+      <c r="L5">
+        <v>2030</v>
+      </c>
+      <c r="M5">
+        <v>2031</v>
+      </c>
+      <c r="N5">
+        <v>2032</v>
+      </c>
+      <c r="O5">
+        <v>2033</v>
+      </c>
+      <c r="P5">
+        <v>2034</v>
+      </c>
+      <c r="Q5">
+        <v>2035</v>
+      </c>
+      <c r="R5">
+        <v>2036</v>
+      </c>
+      <c r="S5">
+        <v>2037</v>
+      </c>
+      <c r="T5">
+        <v>2038</v>
+      </c>
+      <c r="U5">
+        <v>2039</v>
+      </c>
+      <c r="V5">
+        <v>2040</v>
+      </c>
+      <c r="W5">
+        <v>2041</v>
+      </c>
+      <c r="X5">
+        <v>2042</v>
+      </c>
+      <c r="Y5">
+        <v>2043</v>
+      </c>
+      <c r="Z5">
+        <v>2044</v>
+      </c>
+      <c r="AA5">
+        <v>2045</v>
+      </c>
+      <c r="AB5">
+        <v>2046</v>
+      </c>
+      <c r="AC5">
+        <v>2047</v>
+      </c>
+      <c r="AD5">
+        <v>2048</v>
+      </c>
+      <c r="AE5">
+        <v>2049</v>
+      </c>
+      <c r="AF5">
+        <v>2050</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" s="39" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>263</v>
+      </c>
+      <c r="C6" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>146</v>
+      </c>
+      <c r="F6" s="39">
+        <v>21699.671875</v>
+      </c>
+      <c r="G6" s="39">
+        <v>22171.929688</v>
+      </c>
+      <c r="H6" s="39">
+        <v>22685.953125</v>
+      </c>
+      <c r="I6" s="39">
+        <v>23162.595702999999</v>
+      </c>
+      <c r="J6" s="39">
+        <v>23590.015625</v>
+      </c>
+      <c r="K6" s="39">
+        <v>24042.869140999999</v>
+      </c>
+      <c r="L6" s="39">
+        <v>24479.318359000001</v>
+      </c>
+      <c r="M6" s="39">
+        <v>24877.939452999999</v>
+      </c>
+      <c r="N6" s="39">
+        <v>25299.824218999998</v>
+      </c>
+      <c r="O6" s="39">
+        <v>25731.902343999998</v>
+      </c>
+      <c r="P6" s="39">
+        <v>26166.296875</v>
+      </c>
+      <c r="Q6" s="39">
+        <v>26621.835938</v>
+      </c>
+      <c r="R6" s="39">
+        <v>27077.875</v>
+      </c>
+      <c r="S6" s="39">
+        <v>27546.341797000001</v>
+      </c>
+      <c r="T6" s="39">
+        <v>28018.710938</v>
+      </c>
+      <c r="U6" s="39">
+        <v>28503.035156000002</v>
+      </c>
+      <c r="V6" s="39">
+        <v>29003.939452999999</v>
+      </c>
+      <c r="W6" s="39">
+        <v>29486.919922000001</v>
+      </c>
+      <c r="X6" s="39">
+        <v>29991.914062</v>
+      </c>
+      <c r="Y6" s="39">
+        <v>30494.671875</v>
+      </c>
+      <c r="Z6" s="39">
+        <v>30998.292968999998</v>
+      </c>
+      <c r="AA6" s="39">
+        <v>31501.849609000001</v>
+      </c>
+      <c r="AB6" s="39">
+        <v>32021.367188</v>
+      </c>
+      <c r="AC6" s="39">
+        <v>32546.509765999999</v>
+      </c>
+      <c r="AD6" s="39">
+        <v>33074.625</v>
+      </c>
+      <c r="AE6" s="39">
+        <v>33617.65625</v>
+      </c>
+      <c r="AF6" s="39">
+        <v>34162.722655999998</v>
+      </c>
+      <c r="AG6" s="40">
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B8" t="s">
+        <v>260</v>
+      </c>
+      <c r="C8" t="s">
+        <v>259</v>
+      </c>
+      <c r="D8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F8">
+        <v>15151.048828000001</v>
+      </c>
+      <c r="G8">
+        <v>15524.572265999999</v>
+      </c>
+      <c r="H8">
+        <v>15926.875</v>
+      </c>
+      <c r="I8">
+        <v>16368.389648</v>
+      </c>
+      <c r="J8">
+        <v>16790.757812</v>
+      </c>
+      <c r="K8">
+        <v>17202.304688</v>
+      </c>
+      <c r="L8">
+        <v>17601.259765999999</v>
+      </c>
+      <c r="M8">
+        <v>17987.453125</v>
+      </c>
+      <c r="N8">
+        <v>18384.164062</v>
+      </c>
+      <c r="O8">
+        <v>18798.505859000001</v>
+      </c>
+      <c r="P8">
+        <v>19221.488281000002</v>
+      </c>
+      <c r="Q8">
+        <v>19634.119140999999</v>
+      </c>
+      <c r="R8">
+        <v>20038.617188</v>
+      </c>
+      <c r="S8">
+        <v>20454.4375</v>
+      </c>
+      <c r="T8">
+        <v>20860.751952999999</v>
+      </c>
+      <c r="U8">
+        <v>21268.019531000002</v>
+      </c>
+      <c r="V8">
+        <v>21682.087890999999</v>
+      </c>
+      <c r="W8">
+        <v>22091.867188</v>
+      </c>
+      <c r="X8">
+        <v>22505.357422000001</v>
+      </c>
+      <c r="Y8">
+        <v>22920.322265999999</v>
+      </c>
+      <c r="Z8">
+        <v>23337.054688</v>
+      </c>
+      <c r="AA8">
+        <v>23747.720702999999</v>
+      </c>
+      <c r="AB8">
+        <v>24165.929688</v>
+      </c>
+      <c r="AC8">
+        <v>24601.738281000002</v>
+      </c>
+      <c r="AD8">
+        <v>25052.125</v>
+      </c>
+      <c r="AE8">
+        <v>25519.373047000001</v>
+      </c>
+      <c r="AF8">
+        <v>25983.876952999999</v>
+      </c>
+      <c r="AG8" s="38">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>258</v>
+      </c>
+      <c r="B9" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D9" t="s">
+        <v>146</v>
+      </c>
+      <c r="F9">
+        <v>3493.9401859999998</v>
+      </c>
+      <c r="G9">
+        <v>3594.2749020000001</v>
+      </c>
+      <c r="H9">
+        <v>3649.9650879999999</v>
+      </c>
+      <c r="I9">
+        <v>3702.7680660000001</v>
+      </c>
+      <c r="J9">
+        <v>3743.2592770000001</v>
+      </c>
+      <c r="K9">
+        <v>3788.8195799999999</v>
+      </c>
+      <c r="L9">
+        <v>3847.7333979999999</v>
+      </c>
+      <c r="M9">
+        <v>3920.0410160000001</v>
+      </c>
+      <c r="N9">
+        <v>4008.1608890000002</v>
+      </c>
+      <c r="O9">
+        <v>4113.0161129999997</v>
+      </c>
+      <c r="P9">
+        <v>4230.0839839999999</v>
+      </c>
+      <c r="Q9">
+        <v>4347.6567379999997</v>
+      </c>
+      <c r="R9">
+        <v>4442.9697269999997</v>
+      </c>
+      <c r="S9">
+        <v>4543.9965819999998</v>
+      </c>
+      <c r="T9">
+        <v>4646.4091799999997</v>
+      </c>
+      <c r="U9">
+        <v>4749.9125979999999</v>
+      </c>
+      <c r="V9">
+        <v>4858.6166990000002</v>
+      </c>
+      <c r="W9">
+        <v>4967.8120120000003</v>
+      </c>
+      <c r="X9">
+        <v>5077.7265619999998</v>
+      </c>
+      <c r="Y9">
+        <v>5191.7080079999996</v>
+      </c>
+      <c r="Z9">
+        <v>5302.5922849999997</v>
+      </c>
+      <c r="AA9">
+        <v>5413.7685549999997</v>
+      </c>
+      <c r="AB9">
+        <v>5525.9057620000003</v>
+      </c>
+      <c r="AC9">
+        <v>5645.53125</v>
+      </c>
+      <c r="AD9">
+        <v>5763.8344729999999</v>
+      </c>
+      <c r="AE9">
+        <v>5887.2368159999996</v>
+      </c>
+      <c r="AF9">
+        <v>6010.6650390000004</v>
+      </c>
+      <c r="AG9" s="38">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>255</v>
+      </c>
+      <c r="B10" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" t="s">
+        <v>253</v>
+      </c>
+      <c r="D10" t="s">
+        <v>146</v>
+      </c>
+      <c r="F10">
+        <v>3663.0996089999999</v>
+      </c>
+      <c r="G10">
+        <v>3692.658203</v>
+      </c>
+      <c r="H10">
+        <v>3702.429443</v>
+      </c>
+      <c r="I10">
+        <v>3705.2067870000001</v>
+      </c>
+      <c r="J10">
+        <v>3700.4521479999999</v>
+      </c>
+      <c r="K10">
+        <v>3692.9423830000001</v>
+      </c>
+      <c r="L10">
+        <v>3692.6364749999998</v>
+      </c>
+      <c r="M10">
+        <v>3683.7204590000001</v>
+      </c>
+      <c r="N10">
+        <v>3684.8178710000002</v>
+      </c>
+      <c r="O10">
+        <v>3687.0541990000002</v>
+      </c>
+      <c r="P10">
+        <v>3686.1518550000001</v>
+      </c>
+      <c r="Q10">
+        <v>3695.8171390000002</v>
+      </c>
+      <c r="R10">
+        <v>3716.4252929999998</v>
+      </c>
+      <c r="S10">
+        <v>3739.5742190000001</v>
+      </c>
+      <c r="T10">
+        <v>3763.750732</v>
+      </c>
+      <c r="U10">
+        <v>3787.4892580000001</v>
+      </c>
+      <c r="V10">
+        <v>3815.9572750000002</v>
+      </c>
+      <c r="W10">
+        <v>3832.6760250000002</v>
+      </c>
+      <c r="X10">
+        <v>3856.4804690000001</v>
+      </c>
+      <c r="Y10">
+        <v>3879.9494629999999</v>
+      </c>
+      <c r="Z10">
+        <v>3900.8937989999999</v>
+      </c>
+      <c r="AA10">
+        <v>3921.0200199999999</v>
+      </c>
+      <c r="AB10">
+        <v>3941.8579100000002</v>
+      </c>
+      <c r="AC10">
+        <v>3959.2687989999999</v>
+      </c>
+      <c r="AD10">
+        <v>3977.9833979999999</v>
+      </c>
+      <c r="AE10">
+        <v>3997.8740229999999</v>
+      </c>
+      <c r="AF10">
+        <v>4025.7573240000002</v>
+      </c>
+      <c r="AG10" s="38">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>252</v>
+      </c>
+      <c r="B11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C11" t="s">
+        <v>250</v>
+      </c>
+      <c r="D11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F11">
+        <v>2721.9965820000002</v>
+      </c>
+      <c r="G11">
+        <v>2817.2946780000002</v>
+      </c>
+      <c r="H11">
+        <v>2907.773193</v>
+      </c>
+      <c r="I11">
+        <v>3020.0053710000002</v>
+      </c>
+      <c r="J11">
+        <v>3130.0764159999999</v>
+      </c>
+      <c r="K11">
+        <v>3230.9099120000001</v>
+      </c>
+      <c r="L11">
+        <v>3328.4602049999999</v>
+      </c>
+      <c r="M11">
+        <v>3416.2929690000001</v>
+      </c>
+      <c r="N11">
+        <v>3509.2990719999998</v>
+      </c>
+      <c r="O11">
+        <v>3589.1208499999998</v>
+      </c>
+      <c r="P11">
+        <v>3685.4812010000001</v>
+      </c>
+      <c r="Q11">
+        <v>3762.8725589999999</v>
+      </c>
+      <c r="R11">
+        <v>3821.4929200000001</v>
+      </c>
+      <c r="S11">
+        <v>3883.985107</v>
+      </c>
+      <c r="T11">
+        <v>3946.661865</v>
+      </c>
+      <c r="U11">
+        <v>4015.3747560000002</v>
+      </c>
+      <c r="V11">
+        <v>4087.0009770000001</v>
+      </c>
+      <c r="W11">
+        <v>4157.4023440000001</v>
+      </c>
+      <c r="X11">
+        <v>4230.5415039999998</v>
+      </c>
+      <c r="Y11">
+        <v>4302.7900390000004</v>
+      </c>
+      <c r="Z11">
+        <v>4378.001953</v>
+      </c>
+      <c r="AA11">
+        <v>4441.7431640000004</v>
+      </c>
+      <c r="AB11">
+        <v>4512.8193359999996</v>
+      </c>
+      <c r="AC11">
+        <v>4584.1948240000002</v>
+      </c>
+      <c r="AD11">
+        <v>4643.1547849999997</v>
+      </c>
+      <c r="AE11">
+        <v>4699.0834960000002</v>
+      </c>
+      <c r="AF11">
+        <v>4750.3662109999996</v>
+      </c>
+      <c r="AG11" s="38">
+        <v>2.1999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D12" t="s">
+        <v>146</v>
+      </c>
+      <c r="F12">
+        <v>4085.1303710000002</v>
+      </c>
+      <c r="G12">
+        <v>4233.8344729999999</v>
+      </c>
+      <c r="H12">
+        <v>4349.9331050000001</v>
+      </c>
+      <c r="I12">
+        <v>4482.4501950000003</v>
+      </c>
+      <c r="J12">
+        <v>4617.8198240000002</v>
+      </c>
+      <c r="K12">
+        <v>4748.7231449999999</v>
+      </c>
+      <c r="L12">
+        <v>4891.5942379999997</v>
+      </c>
+      <c r="M12">
+        <v>5038.9599609999996</v>
+      </c>
+      <c r="N12">
+        <v>5209.8481449999999</v>
+      </c>
+      <c r="O12">
+        <v>5367.5698240000002</v>
+      </c>
+      <c r="P12">
+        <v>5568.1762699999999</v>
+      </c>
+      <c r="Q12">
+        <v>5712.3798829999996</v>
+      </c>
+      <c r="R12">
+        <v>5821.236328</v>
+      </c>
+      <c r="S12">
+        <v>5943.6083980000003</v>
+      </c>
+      <c r="T12">
+        <v>6033.5253910000001</v>
+      </c>
+      <c r="U12">
+        <v>6125.2973629999997</v>
+      </c>
+      <c r="V12">
+        <v>6213.2670900000003</v>
+      </c>
+      <c r="W12">
+        <v>6286.7270509999998</v>
+      </c>
+      <c r="X12">
+        <v>6369.7358400000003</v>
+      </c>
+      <c r="Y12">
+        <v>6443.5234380000002</v>
+      </c>
+      <c r="Z12">
+        <v>6522.7333980000003</v>
+      </c>
+      <c r="AA12">
+        <v>6587.8569340000004</v>
+      </c>
+      <c r="AB12">
+        <v>6664.9497069999998</v>
+      </c>
+      <c r="AC12">
+        <v>6768.4184569999998</v>
+      </c>
+      <c r="AD12">
+        <v>6865.8984380000002</v>
+      </c>
+      <c r="AE12">
+        <v>6979.140625</v>
+      </c>
+      <c r="AF12">
+        <v>7082.5068359999996</v>
+      </c>
+      <c r="AG12" s="38">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" t="s">
+        <v>244</v>
+      </c>
+      <c r="C15" t="s">
+        <v>243</v>
+      </c>
+      <c r="D15" t="s">
+        <v>239</v>
+      </c>
+      <c r="F15">
+        <v>3.4284460000000001</v>
+      </c>
+      <c r="G15">
+        <v>3.411206</v>
+      </c>
+      <c r="H15">
+        <v>3.3420169999999998</v>
+      </c>
+      <c r="I15">
+        <v>3.275083</v>
+      </c>
+      <c r="J15">
+        <v>3.2179419999999999</v>
+      </c>
+      <c r="K15">
+        <v>3.1543049999999999</v>
+      </c>
+      <c r="L15">
+        <v>3.0912160000000002</v>
+      </c>
+      <c r="M15">
+        <v>3.032044</v>
+      </c>
+      <c r="N15">
+        <v>2.9704809999999999</v>
+      </c>
+      <c r="O15">
+        <v>2.9045879999999999</v>
+      </c>
+      <c r="P15">
+        <v>2.8461699999999999</v>
+      </c>
+      <c r="Q15">
+        <v>2.7882769999999999</v>
+      </c>
+      <c r="R15">
+        <v>2.7347980000000001</v>
+      </c>
+      <c r="S15">
+        <v>2.6815500000000001</v>
+      </c>
+      <c r="T15">
+        <v>2.6327989999999999</v>
+      </c>
+      <c r="U15">
+        <v>2.587637</v>
+      </c>
+      <c r="V15">
+        <v>2.5466350000000002</v>
+      </c>
+      <c r="W15">
+        <v>2.5057239999999998</v>
+      </c>
+      <c r="X15">
+        <v>2.464391</v>
+      </c>
+      <c r="Y15">
+        <v>2.4268930000000002</v>
+      </c>
+      <c r="Z15">
+        <v>2.392449</v>
+      </c>
+      <c r="AA15">
+        <v>2.3607740000000002</v>
+      </c>
+      <c r="AB15">
+        <v>2.328157</v>
+      </c>
+      <c r="AC15">
+        <v>2.3003429999999998</v>
+      </c>
+      <c r="AD15">
+        <v>2.2698969999999998</v>
+      </c>
+      <c r="AE15">
+        <v>2.2427670000000002</v>
+      </c>
+      <c r="AF15">
+        <v>2.216291</v>
+      </c>
+      <c r="AG15" s="38">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>242</v>
+      </c>
+      <c r="B16" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" t="s">
+        <v>240</v>
+      </c>
+      <c r="D16" t="s">
+        <v>239</v>
+      </c>
+      <c r="F16">
+        <v>4.3222800000000001</v>
+      </c>
+      <c r="G16">
+        <v>4.2643950000000004</v>
+      </c>
+      <c r="H16">
+        <v>4.132428</v>
+      </c>
+      <c r="I16">
+        <v>4.0300190000000002</v>
+      </c>
+      <c r="J16">
+        <v>3.951152</v>
+      </c>
+      <c r="K16">
+        <v>3.8704619999999998</v>
+      </c>
+      <c r="L16">
+        <v>3.7755049999999999</v>
+      </c>
+      <c r="M16">
+        <v>3.6931050000000001</v>
+      </c>
+      <c r="N16">
+        <v>3.5904980000000002</v>
+      </c>
+      <c r="O16">
+        <v>3.5060579999999999</v>
+      </c>
+      <c r="P16">
+        <v>3.4292720000000001</v>
+      </c>
+      <c r="Q16">
+        <v>3.3496980000000001</v>
+      </c>
+      <c r="R16">
+        <v>3.2760120000000001</v>
+      </c>
+      <c r="S16">
+        <v>3.1973530000000001</v>
+      </c>
+      <c r="T16">
+        <v>3.1336360000000001</v>
+      </c>
+      <c r="U16">
+        <v>3.0601430000000001</v>
+      </c>
+      <c r="V16">
+        <v>3.011317</v>
+      </c>
+      <c r="W16">
+        <v>2.9696039999999999</v>
+      </c>
+      <c r="X16">
+        <v>2.9267889999999999</v>
+      </c>
+      <c r="Y16">
+        <v>2.8854329999999999</v>
+      </c>
+      <c r="Z16">
+        <v>2.8475579999999998</v>
+      </c>
+      <c r="AA16">
+        <v>2.8097159999999999</v>
+      </c>
+      <c r="AB16">
+        <v>2.7706499999999998</v>
+      </c>
+      <c r="AC16">
+        <v>2.7378589999999998</v>
+      </c>
+      <c r="AD16">
+        <v>2.7034189999999998</v>
+      </c>
+      <c r="AE16">
+        <v>2.6727750000000001</v>
+      </c>
+      <c r="AF16">
+        <v>2.6398160000000002</v>
+      </c>
+      <c r="AG16" s="38">
+        <v>-1.9E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>238</v>
+      </c>
+      <c r="B18" t="s">
+        <v>237</v>
+      </c>
+      <c r="C18" t="s">
+        <v>236</v>
+      </c>
+      <c r="D18" t="s">
+        <v>235</v>
+      </c>
+      <c r="F18">
+        <v>1.3431169999999999</v>
+      </c>
+      <c r="G18">
+        <v>1.37063</v>
+      </c>
+      <c r="H18">
+        <v>1.3938109999999999</v>
+      </c>
+      <c r="I18">
+        <v>1.4171339999999999</v>
+      </c>
+      <c r="J18">
+        <v>1.443964</v>
+      </c>
+      <c r="K18">
+        <v>1.4697340000000001</v>
+      </c>
+      <c r="L18">
+        <v>1.497355</v>
+      </c>
+      <c r="M18">
+        <v>1.528316</v>
+      </c>
+      <c r="N18">
+        <v>1.5609390000000001</v>
+      </c>
+      <c r="O18">
+        <v>1.5951900000000001</v>
+      </c>
+      <c r="P18">
+        <v>1.6307860000000001</v>
+      </c>
+      <c r="Q18">
+        <v>1.666277</v>
+      </c>
+      <c r="R18">
+        <v>1.700817</v>
+      </c>
+      <c r="S18">
+        <v>1.736221</v>
+      </c>
+      <c r="T18">
+        <v>1.7723930000000001</v>
+      </c>
+      <c r="U18">
+        <v>1.808899</v>
+      </c>
+      <c r="V18">
+        <v>1.8468249999999999</v>
+      </c>
+      <c r="W18">
+        <v>1.8862300000000001</v>
+      </c>
+      <c r="X18">
+        <v>1.9269259999999999</v>
+      </c>
+      <c r="Y18">
+        <v>1.9691639999999999</v>
+      </c>
+      <c r="Z18">
+        <v>2.0126740000000001</v>
+      </c>
+      <c r="AA18">
+        <v>2.0575079999999999</v>
+      </c>
+      <c r="AB18">
+        <v>2.1034350000000002</v>
+      </c>
+      <c r="AC18">
+        <v>2.151106</v>
+      </c>
+      <c r="AD18">
+        <v>2.200072</v>
+      </c>
+      <c r="AE18">
+        <v>2.2503690000000001</v>
+      </c>
+      <c r="AF18">
+        <v>2.3020529999999999</v>
+      </c>
+      <c r="AG18" s="38">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>233</v>
+      </c>
+      <c r="B20" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" t="s">
+        <v>231</v>
+      </c>
+      <c r="D20" t="s">
+        <v>227</v>
+      </c>
+      <c r="F20">
+        <v>3.1332360000000001</v>
+      </c>
+      <c r="G20">
+        <v>3.1873100000000001</v>
+      </c>
+      <c r="H20">
+        <v>3.2438159999999998</v>
+      </c>
+      <c r="I20">
+        <v>3.29739</v>
+      </c>
+      <c r="J20">
+        <v>3.358501</v>
+      </c>
+      <c r="K20">
+        <v>3.4197440000000001</v>
+      </c>
+      <c r="L20">
+        <v>3.4840200000000001</v>
+      </c>
+      <c r="M20">
+        <v>3.5537990000000002</v>
+      </c>
+      <c r="N20">
+        <v>3.6269870000000002</v>
+      </c>
+      <c r="O20">
+        <v>3.70384</v>
+      </c>
+      <c r="P20">
+        <v>3.783029</v>
+      </c>
+      <c r="Q20">
+        <v>3.8627280000000002</v>
+      </c>
+      <c r="R20">
+        <v>3.9415480000000001</v>
+      </c>
+      <c r="S20">
+        <v>4.0227899999999996</v>
+      </c>
+      <c r="T20">
+        <v>4.1064660000000002</v>
+      </c>
+      <c r="U20">
+        <v>4.1913130000000001</v>
+      </c>
+      <c r="V20">
+        <v>4.2789830000000002</v>
+      </c>
+      <c r="W20">
+        <v>4.3724210000000001</v>
+      </c>
+      <c r="X20">
+        <v>4.4684990000000004</v>
+      </c>
+      <c r="Y20">
+        <v>4.5693440000000001</v>
+      </c>
+      <c r="Z20">
+        <v>4.672993</v>
+      </c>
+      <c r="AA20">
+        <v>4.780564</v>
+      </c>
+      <c r="AB20">
+        <v>4.8909840000000004</v>
+      </c>
+      <c r="AC20">
+        <v>5.0057999999999998</v>
+      </c>
+      <c r="AD20">
+        <v>5.1239569999999999</v>
+      </c>
+      <c r="AE20">
+        <v>5.2466879999999998</v>
+      </c>
+      <c r="AF20">
+        <v>5.3733490000000002</v>
+      </c>
+      <c r="AG20" s="38">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>230</v>
+      </c>
+      <c r="B21" t="s">
+        <v>229</v>
+      </c>
+      <c r="C21" t="s">
+        <v>228</v>
+      </c>
+      <c r="D21" t="s">
+        <v>227</v>
+      </c>
+      <c r="F21">
+        <v>2.7925080000000002</v>
+      </c>
+      <c r="G21">
+        <v>2.6914549999999999</v>
+      </c>
+      <c r="H21">
+        <v>2.6876129999999998</v>
+      </c>
+      <c r="I21">
+        <v>2.6521680000000001</v>
+      </c>
+      <c r="J21">
+        <v>2.6949160000000001</v>
+      </c>
+      <c r="K21">
+        <v>2.7545130000000002</v>
+      </c>
+      <c r="L21">
+        <v>2.8223549999999999</v>
+      </c>
+      <c r="M21">
+        <v>2.9040720000000002</v>
+      </c>
+      <c r="N21">
+        <v>2.9858380000000002</v>
+      </c>
+      <c r="O21">
+        <v>3.0742289999999999</v>
+      </c>
+      <c r="P21">
+        <v>3.1541549999999998</v>
+      </c>
+      <c r="Q21">
+        <v>3.2223570000000001</v>
+      </c>
+      <c r="R21">
+        <v>3.2833749999999999</v>
+      </c>
+      <c r="S21">
+        <v>3.3454839999999999</v>
+      </c>
+      <c r="T21">
+        <v>3.4118200000000001</v>
+      </c>
+      <c r="U21">
+        <v>3.4737680000000002</v>
+      </c>
+      <c r="V21">
+        <v>3.537099</v>
+      </c>
+      <c r="W21">
+        <v>3.624193</v>
+      </c>
+      <c r="X21">
+        <v>3.7039749999999998</v>
+      </c>
+      <c r="Y21">
+        <v>3.798629</v>
+      </c>
+      <c r="Z21">
+        <v>3.8853330000000001</v>
+      </c>
+      <c r="AA21">
+        <v>3.978532</v>
+      </c>
+      <c r="AB21">
+        <v>4.0711120000000003</v>
+      </c>
+      <c r="AC21">
+        <v>4.1738499999999998</v>
+      </c>
+      <c r="AD21">
+        <v>4.2806730000000002</v>
+      </c>
+      <c r="AE21">
+        <v>4.4049050000000003</v>
+      </c>
+      <c r="AF21">
+        <v>4.5420879999999997</v>
+      </c>
+      <c r="AG21" s="38">
+        <v>1.9E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>225</v>
+      </c>
+      <c r="B23" t="s">
+        <v>224</v>
+      </c>
+      <c r="C23" t="s">
+        <v>223</v>
+      </c>
+      <c r="D23" t="s">
+        <v>213</v>
+      </c>
+      <c r="F23">
+        <v>2.5444830000000001</v>
+      </c>
+      <c r="G23">
+        <v>2.5369220000000001</v>
+      </c>
+      <c r="H23">
+        <v>2.5284499999999999</v>
+      </c>
+      <c r="I23">
+        <v>2.5255619999999999</v>
+      </c>
+      <c r="J23">
+        <v>2.550341</v>
+      </c>
+      <c r="K23">
+        <v>2.579834</v>
+      </c>
+      <c r="L23">
+        <v>2.6191559999999998</v>
+      </c>
+      <c r="M23">
+        <v>2.6681780000000002</v>
+      </c>
+      <c r="N23">
+        <v>2.726175</v>
+      </c>
+      <c r="O23">
+        <v>2.7891460000000001</v>
+      </c>
+      <c r="P23">
+        <v>2.8477459999999999</v>
+      </c>
+      <c r="Q23">
+        <v>2.8974600000000001</v>
+      </c>
+      <c r="R23">
+        <v>2.9412569999999998</v>
+      </c>
+      <c r="S23">
+        <v>2.990532</v>
+      </c>
+      <c r="T23">
+        <v>3.0430139999999999</v>
+      </c>
+      <c r="U23">
+        <v>3.0926149999999999</v>
+      </c>
+      <c r="V23">
+        <v>3.145597</v>
+      </c>
+      <c r="W23">
+        <v>3.2068669999999999</v>
+      </c>
+      <c r="X23">
+        <v>3.2677420000000001</v>
+      </c>
+      <c r="Y23">
+        <v>3.331159</v>
+      </c>
+      <c r="Z23">
+        <v>3.3918210000000002</v>
+      </c>
+      <c r="AA23">
+        <v>3.4568500000000002</v>
+      </c>
+      <c r="AB23">
+        <v>3.5212629999999998</v>
+      </c>
+      <c r="AC23">
+        <v>3.5894659999999998</v>
+      </c>
+      <c r="AD23">
+        <v>3.660784</v>
+      </c>
+      <c r="AE23">
+        <v>3.7397339999999999</v>
+      </c>
+      <c r="AF23">
+        <v>3.8224320000000001</v>
+      </c>
+      <c r="AG23" s="38">
+        <v>1.6E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>222</v>
+      </c>
+      <c r="B24" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" t="s">
+        <v>220</v>
+      </c>
+      <c r="D24" t="s">
+        <v>213</v>
+      </c>
+      <c r="F24">
+        <v>2.310759</v>
+      </c>
+      <c r="G24">
+        <v>2.3202950000000002</v>
+      </c>
+      <c r="H24">
+        <v>2.3035570000000001</v>
+      </c>
+      <c r="I24">
+        <v>2.2750270000000001</v>
+      </c>
+      <c r="J24">
+        <v>2.3186619999999998</v>
+      </c>
+      <c r="K24">
+        <v>2.3827029999999998</v>
+      </c>
+      <c r="L24">
+        <v>2.4596049999999998</v>
+      </c>
+      <c r="M24">
+        <v>2.5416979999999998</v>
+      </c>
+      <c r="N24">
+        <v>2.6475369999999998</v>
+      </c>
+      <c r="O24">
+        <v>2.7716880000000002</v>
+      </c>
+      <c r="P24">
+        <v>2.8764110000000001</v>
+      </c>
+      <c r="Q24">
+        <v>2.9504220000000001</v>
+      </c>
+      <c r="R24">
+        <v>3.007536</v>
+      </c>
+      <c r="S24">
+        <v>3.0685519999999999</v>
+      </c>
+      <c r="T24">
+        <v>3.1362619999999999</v>
+      </c>
+      <c r="U24">
+        <v>3.1936040000000001</v>
+      </c>
+      <c r="V24">
+        <v>3.256008</v>
+      </c>
+      <c r="W24">
+        <v>3.3452799999999998</v>
+      </c>
+      <c r="X24">
+        <v>3.4294229999999999</v>
+      </c>
+      <c r="Y24">
+        <v>3.5230860000000002</v>
+      </c>
+      <c r="Z24">
+        <v>3.6022310000000002</v>
+      </c>
+      <c r="AA24">
+        <v>3.6951930000000002</v>
+      </c>
+      <c r="AB24">
+        <v>3.7813189999999999</v>
+      </c>
+      <c r="AC24">
+        <v>3.8727140000000002</v>
+      </c>
+      <c r="AD24">
+        <v>3.9718249999999999</v>
+      </c>
+      <c r="AE24">
+        <v>4.0962160000000001</v>
+      </c>
+      <c r="AF24">
+        <v>4.2370239999999999</v>
+      </c>
+      <c r="AG24" s="38">
+        <v>2.4E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>219</v>
+      </c>
+      <c r="B25" t="s">
+        <v>218</v>
+      </c>
+      <c r="C25" t="s">
+        <v>217</v>
+      </c>
+      <c r="D25" t="s">
+        <v>213</v>
+      </c>
+      <c r="F25">
+        <v>3.0321470000000001</v>
+      </c>
+      <c r="G25">
+        <v>2.8606750000000001</v>
+      </c>
+      <c r="H25">
+        <v>2.7882159999999998</v>
+      </c>
+      <c r="I25">
+        <v>2.7634050000000001</v>
+      </c>
+      <c r="J25">
+        <v>2.74133</v>
+      </c>
+      <c r="K25">
+        <v>2.739916</v>
+      </c>
+      <c r="L25">
+        <v>2.7641249999999999</v>
+      </c>
+      <c r="M25">
+        <v>2.8123089999999999</v>
+      </c>
+      <c r="N25">
+        <v>2.8618760000000001</v>
+      </c>
+      <c r="O25">
+        <v>2.9031259999999999</v>
+      </c>
+      <c r="P25">
+        <v>2.9436629999999999</v>
+      </c>
+      <c r="Q25">
+        <v>2.9681030000000002</v>
+      </c>
+      <c r="R25">
+        <v>2.9973230000000002</v>
+      </c>
+      <c r="S25">
+        <v>3.0429599999999999</v>
+      </c>
+      <c r="T25">
+        <v>3.0893760000000001</v>
+      </c>
+      <c r="U25">
+        <v>3.1330010000000001</v>
+      </c>
+      <c r="V25">
+        <v>3.182893</v>
+      </c>
+      <c r="W25">
+        <v>3.233063</v>
+      </c>
+      <c r="X25">
+        <v>3.2827130000000002</v>
+      </c>
+      <c r="Y25">
+        <v>3.3297669999999999</v>
+      </c>
+      <c r="Z25">
+        <v>3.375909</v>
+      </c>
+      <c r="AA25">
+        <v>3.4205899999999998</v>
+      </c>
+      <c r="AB25">
+        <v>3.4675090000000002</v>
+      </c>
+      <c r="AC25">
+        <v>3.520473</v>
+      </c>
+      <c r="AD25">
+        <v>3.5745100000000001</v>
+      </c>
+      <c r="AE25">
+        <v>3.6313430000000002</v>
+      </c>
+      <c r="AF25">
+        <v>3.6830430000000001</v>
+      </c>
+      <c r="AG25" s="38">
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" t="s">
+        <v>215</v>
+      </c>
+      <c r="C26" t="s">
+        <v>214</v>
+      </c>
+      <c r="D26" t="s">
+        <v>213</v>
+      </c>
+      <c r="F26">
+        <v>2.5845829999999999</v>
+      </c>
+      <c r="G26">
+        <v>2.5789309999999999</v>
+      </c>
+      <c r="H26">
+        <v>2.570989</v>
+      </c>
+      <c r="I26">
+        <v>2.5752169999999999</v>
+      </c>
+      <c r="J26">
+        <v>2.5917110000000001</v>
+      </c>
+      <c r="K26">
+        <v>2.6081340000000002</v>
+      </c>
+      <c r="L26">
+        <v>2.6363020000000001</v>
+      </c>
+      <c r="M26">
+        <v>2.6758570000000002</v>
+      </c>
+      <c r="N26">
+        <v>2.7211020000000001</v>
+      </c>
+      <c r="O26">
+        <v>2.768586</v>
+      </c>
+      <c r="P26">
+        <v>2.817564</v>
+      </c>
+      <c r="Q26">
+        <v>2.8628550000000001</v>
+      </c>
+      <c r="R26">
+        <v>2.9047350000000001</v>
+      </c>
+      <c r="S26">
+        <v>2.9532609999999999</v>
+      </c>
+      <c r="T26">
+        <v>3.0041820000000001</v>
+      </c>
+      <c r="U26">
+        <v>3.0542050000000001</v>
+      </c>
+      <c r="V26">
+        <v>3.1074130000000002</v>
+      </c>
+      <c r="W26">
+        <v>3.1637219999999999</v>
+      </c>
+      <c r="X26">
+        <v>3.2208929999999998</v>
+      </c>
+      <c r="Y26">
+        <v>3.2785319999999998</v>
+      </c>
+      <c r="Z26">
+        <v>3.3365719999999999</v>
+      </c>
+      <c r="AA26">
+        <v>3.3964110000000001</v>
+      </c>
+      <c r="AB26">
+        <v>3.457436</v>
+      </c>
+      <c r="AC26">
+        <v>3.522192</v>
+      </c>
+      <c r="AD26">
+        <v>3.5888740000000001</v>
+      </c>
+      <c r="AE26">
+        <v>3.6585109999999998</v>
+      </c>
+      <c r="AF26">
+        <v>3.728199</v>
+      </c>
+      <c r="AG26" s="38">
+        <v>1.4E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>210</v>
+      </c>
+      <c r="B28" t="s">
+        <v>209</v>
+      </c>
+      <c r="C28" t="s">
+        <v>208</v>
+      </c>
+      <c r="D28" t="s">
+        <v>201</v>
+      </c>
+      <c r="F28">
+        <v>5.145988</v>
+      </c>
+      <c r="G28">
+        <v>3.788913</v>
+      </c>
+      <c r="H28">
+        <v>2.6381709999999998</v>
+      </c>
+      <c r="I28">
+        <v>2.6231360000000001</v>
+      </c>
+      <c r="J28">
+        <v>2.6236510000000002</v>
+      </c>
+      <c r="K28">
+        <v>2.6241110000000001</v>
+      </c>
+      <c r="L28">
+        <v>2.6239669999999999</v>
+      </c>
+      <c r="M28">
+        <v>2.6230159999999998</v>
+      </c>
+      <c r="N28">
+        <v>2.6237149999999998</v>
+      </c>
+      <c r="O28">
+        <v>2.6252110000000002</v>
+      </c>
+      <c r="P28">
+        <v>2.62642</v>
+      </c>
+      <c r="Q28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="R28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="S28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="T28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="U28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="V28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="W28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="X28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="Y28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="Z28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AA28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AB28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AC28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AD28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AE28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AF28">
+        <v>2.6271279999999999</v>
+      </c>
+      <c r="AG28" s="38">
+        <v>-2.5999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" t="s">
+        <v>206</v>
+      </c>
+      <c r="C29" t="s">
+        <v>205</v>
+      </c>
+      <c r="D29" t="s">
+        <v>201</v>
+      </c>
+      <c r="F29">
+        <v>4.0761909999999997</v>
+      </c>
+      <c r="G29">
+        <v>3.4812539999999998</v>
+      </c>
+      <c r="H29">
+        <v>3.2802570000000002</v>
+      </c>
+      <c r="I29">
+        <v>3.187414</v>
+      </c>
+      <c r="J29">
+        <v>3.1661350000000001</v>
+      </c>
+      <c r="K29">
+        <v>3.1823890000000001</v>
+      </c>
+      <c r="L29">
+        <v>3.2130740000000002</v>
+      </c>
+      <c r="M29">
+        <v>3.2357770000000001</v>
+      </c>
+      <c r="N29">
+        <v>3.2451759999999998</v>
+      </c>
+      <c r="O29">
+        <v>3.2456399999999999</v>
+      </c>
+      <c r="P29">
+        <v>3.2573110000000001</v>
+      </c>
+      <c r="Q29">
+        <v>3.2711830000000002</v>
+      </c>
+      <c r="R29">
+        <v>3.280437</v>
+      </c>
+      <c r="S29">
+        <v>3.281555</v>
+      </c>
+      <c r="T29">
+        <v>3.27677</v>
+      </c>
+      <c r="U29">
+        <v>3.2741150000000001</v>
+      </c>
+      <c r="V29">
+        <v>3.2669990000000002</v>
+      </c>
+      <c r="W29">
+        <v>3.2605599999999999</v>
+      </c>
+      <c r="X29">
+        <v>3.2607439999999999</v>
+      </c>
+      <c r="Y29">
+        <v>3.2648700000000002</v>
+      </c>
+      <c r="Z29">
+        <v>3.2731889999999999</v>
+      </c>
+      <c r="AA29">
+        <v>3.280186</v>
+      </c>
+      <c r="AB29">
+        <v>3.2903340000000001</v>
+      </c>
+      <c r="AC29">
+        <v>3.30423</v>
+      </c>
+      <c r="AD29">
+        <v>3.309904</v>
+      </c>
+      <c r="AE29">
+        <v>3.3122959999999999</v>
+      </c>
+      <c r="AF29">
+        <v>3.3176429999999999</v>
+      </c>
+      <c r="AG29" s="38">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>204</v>
+      </c>
+      <c r="B30" t="s">
+        <v>203</v>
+      </c>
+      <c r="C30" t="s">
+        <v>202</v>
+      </c>
+      <c r="D30" t="s">
+        <v>201</v>
+      </c>
+      <c r="F30">
+        <v>5.3953499999999996</v>
+      </c>
+      <c r="G30">
+        <v>5.2155269999999998</v>
+      </c>
+      <c r="H30">
+        <v>5.1328880000000003</v>
+      </c>
+      <c r="I30">
+        <v>5.0468950000000001</v>
+      </c>
+      <c r="J30">
+        <v>5.0313189999999999</v>
+      </c>
+      <c r="K30">
+        <v>5.0189380000000003</v>
+      </c>
+      <c r="L30">
+        <v>5.0012819999999998</v>
+      </c>
+      <c r="M30">
+        <v>4.9834290000000001</v>
+      </c>
+      <c r="N30">
+        <v>4.9927099999999998</v>
+      </c>
+      <c r="O30">
+        <v>5.0253410000000001</v>
+      </c>
+      <c r="P30">
+        <v>5.0341940000000003</v>
+      </c>
+      <c r="Q30">
+        <v>5.057391</v>
+      </c>
+      <c r="R30">
+        <v>5.0617619999999999</v>
+      </c>
+      <c r="S30">
+        <v>5.0389290000000004</v>
+      </c>
+      <c r="T30">
+        <v>5.0397299999999996</v>
+      </c>
+      <c r="U30">
+        <v>5.0290059999999999</v>
+      </c>
+      <c r="V30">
+        <v>4.991193</v>
+      </c>
+      <c r="W30">
+        <v>4.9822199999999999</v>
+      </c>
+      <c r="X30">
+        <v>4.9792139999999998</v>
+      </c>
+      <c r="Y30">
+        <v>4.9968620000000001</v>
+      </c>
+      <c r="Z30">
+        <v>4.9914110000000003</v>
+      </c>
+      <c r="AA30">
+        <v>5.0237999999999996</v>
+      </c>
+      <c r="AB30">
+        <v>5.0331960000000002</v>
+      </c>
+      <c r="AC30">
+        <v>5.0482810000000002</v>
+      </c>
+      <c r="AD30">
+        <v>5.0383800000000001</v>
+      </c>
+      <c r="AE30">
+        <v>5.04697</v>
+      </c>
+      <c r="AF30">
+        <v>5.0879380000000003</v>
+      </c>
+      <c r="AG30" s="38">
+        <v>-2E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>200</v>
+      </c>
+      <c r="B32" t="s">
+        <v>199</v>
+      </c>
+      <c r="C32" t="s">
+        <v>198</v>
+      </c>
+      <c r="D32" t="s">
+        <v>178</v>
+      </c>
+      <c r="F32">
+        <v>28226.228515999999</v>
+      </c>
+      <c r="G32">
+        <v>28832.503906000002</v>
+      </c>
+      <c r="H32">
+        <v>29531.828125</v>
+      </c>
+      <c r="I32">
+        <v>30358.589843999998</v>
+      </c>
+      <c r="J32">
+        <v>31193.046875</v>
+      </c>
+      <c r="K32">
+        <v>31916.195312</v>
+      </c>
+      <c r="L32">
+        <v>32552.964843999998</v>
+      </c>
+      <c r="M32">
+        <v>33193.347655999998</v>
+      </c>
+      <c r="N32">
+        <v>33870.484375</v>
+      </c>
+      <c r="O32">
+        <v>34561.386719000002</v>
+      </c>
+      <c r="P32">
+        <v>35260.015625</v>
+      </c>
+      <c r="Q32">
+        <v>35955.832030999998</v>
+      </c>
+      <c r="R32">
+        <v>36628.492187999997</v>
+      </c>
+      <c r="S32">
+        <v>37306.128905999998</v>
+      </c>
+      <c r="T32">
+        <v>37972.011719000002</v>
+      </c>
+      <c r="U32">
+        <v>38639.6875</v>
+      </c>
+      <c r="V32">
+        <v>39328.714844000002</v>
+      </c>
+      <c r="W32">
+        <v>40017.15625</v>
+      </c>
+      <c r="X32">
+        <v>40711.210937999997</v>
+      </c>
+      <c r="Y32">
+        <v>41405.953125</v>
+      </c>
+      <c r="Z32">
+        <v>42105.753905999998</v>
+      </c>
+      <c r="AA32">
+        <v>42813.265625</v>
+      </c>
+      <c r="AB32">
+        <v>43534.359375</v>
+      </c>
+      <c r="AC32">
+        <v>44293.554687999997</v>
+      </c>
+      <c r="AD32">
+        <v>45075.363280999998</v>
+      </c>
+      <c r="AE32">
+        <v>45888.054687999997</v>
+      </c>
+      <c r="AF32">
+        <v>46699.144530999998</v>
+      </c>
+      <c r="AG32" s="38">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>197</v>
+      </c>
+      <c r="B33" t="s">
+        <v>196</v>
+      </c>
+      <c r="C33" t="s">
+        <v>195</v>
+      </c>
+      <c r="D33" t="s">
+        <v>178</v>
+      </c>
+      <c r="F33">
+        <v>8693.2148440000001</v>
+      </c>
+      <c r="G33">
+        <v>8880.0214840000008</v>
+      </c>
+      <c r="H33">
+        <v>9023.890625</v>
+      </c>
+      <c r="I33">
+        <v>9136.9658199999994</v>
+      </c>
+      <c r="J33">
+        <v>9250.2949219999991</v>
+      </c>
+      <c r="K33">
+        <v>9368.2050780000009</v>
+      </c>
+      <c r="L33">
+        <v>9471.4042969999991</v>
+      </c>
+      <c r="M33">
+        <v>9544.3271480000003</v>
+      </c>
+      <c r="N33">
+        <v>9631.375</v>
+      </c>
+      <c r="O33">
+        <v>9680.8300780000009</v>
+      </c>
+      <c r="P33">
+        <v>9759.0693360000005</v>
+      </c>
+      <c r="Q33">
+        <v>9833.1796880000002</v>
+      </c>
+      <c r="R33">
+        <v>9910.9326170000004</v>
+      </c>
+      <c r="S33">
+        <v>9985.4941409999992</v>
+      </c>
+      <c r="T33">
+        <v>10063.265625</v>
+      </c>
+      <c r="U33">
+        <v>10146.550781</v>
+      </c>
+      <c r="V33">
+        <v>10240.190430000001</v>
+      </c>
+      <c r="W33">
+        <v>10320.269531</v>
+      </c>
+      <c r="X33">
+        <v>10409.382812</v>
+      </c>
+      <c r="Y33">
+        <v>10482.778319999999</v>
+      </c>
+      <c r="Z33">
+        <v>10564.851562</v>
+      </c>
+      <c r="AA33">
+        <v>10653.480469</v>
+      </c>
+      <c r="AB33">
+        <v>10756.961914</v>
+      </c>
+      <c r="AC33">
+        <v>10868.238281</v>
+      </c>
+      <c r="AD33">
+        <v>10969.666992</v>
+      </c>
+      <c r="AE33">
+        <v>11079.728515999999</v>
+      </c>
+      <c r="AF33">
+        <v>11173.776367</v>
+      </c>
+      <c r="AG33" s="38">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>194</v>
+      </c>
+      <c r="B34" t="s">
+        <v>193</v>
+      </c>
+      <c r="C34" t="s">
+        <v>192</v>
+      </c>
+      <c r="D34" t="s">
+        <v>191</v>
+      </c>
+      <c r="E34" t="s">
+        <v>190</v>
+      </c>
+      <c r="F34" t="s">
+        <v>178</v>
+      </c>
+      <c r="H34">
+        <v>2718.2504880000001</v>
+      </c>
+      <c r="I34">
+        <v>2777.9179690000001</v>
+      </c>
+      <c r="J34">
+        <v>2803.5085450000001</v>
+      </c>
+      <c r="K34">
+        <v>2839.2778320000002</v>
+      </c>
+      <c r="L34">
+        <v>2891.1875</v>
+      </c>
+      <c r="M34">
+        <v>2948.4794919999999</v>
+      </c>
+      <c r="N34">
+        <v>2992.1098630000001</v>
+      </c>
+      <c r="O34">
+        <v>3020.3398440000001</v>
+      </c>
+      <c r="P34">
+        <v>3053.4860840000001</v>
+      </c>
+      <c r="Q34">
+        <v>3066.1999510000001</v>
+      </c>
+      <c r="R34">
+        <v>3074.7314449999999</v>
+      </c>
+      <c r="S34">
+        <v>3093.0898440000001</v>
+      </c>
+      <c r="T34">
+        <v>3117.248047</v>
+      </c>
+      <c r="U34">
+        <v>3128.8452149999998</v>
+      </c>
+      <c r="V34">
+        <v>3144.9645999999998</v>
+      </c>
+      <c r="W34">
+        <v>3159.154297</v>
+      </c>
+      <c r="X34">
+        <v>3177.1713869999999</v>
+      </c>
+      <c r="Y34">
+        <v>3191.8076169999999</v>
+      </c>
+      <c r="Z34">
+        <v>3212.5195309999999</v>
+      </c>
+      <c r="AA34">
+        <v>3226.1708979999999</v>
+      </c>
+      <c r="AB34">
+        <v>3241.9814449999999</v>
+      </c>
+      <c r="AC34">
+        <v>3269.1503910000001</v>
+      </c>
+      <c r="AD34">
+        <v>3302.4121089999999</v>
+      </c>
+      <c r="AE34">
+        <v>3332.982422</v>
+      </c>
+      <c r="AF34">
+        <v>3363.429443</v>
+      </c>
+      <c r="AG34">
+        <v>3398.2006839999999</v>
+      </c>
+      <c r="AH34">
+        <v>3430.1721189999998</v>
+      </c>
+      <c r="AI34" s="38">
+        <v>8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C35" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" t="s">
+        <v>178</v>
+      </c>
+      <c r="F35">
+        <v>5974.9643550000001</v>
+      </c>
+      <c r="G35">
+        <v>6102.1030270000001</v>
+      </c>
+      <c r="H35">
+        <v>6220.3818359999996</v>
+      </c>
+      <c r="I35">
+        <v>6297.6884769999997</v>
+      </c>
+      <c r="J35">
+        <v>6359.1064450000003</v>
+      </c>
+      <c r="K35">
+        <v>6419.7250979999999</v>
+      </c>
+      <c r="L35">
+        <v>6479.2939450000003</v>
+      </c>
+      <c r="M35">
+        <v>6523.9873049999997</v>
+      </c>
+      <c r="N35">
+        <v>6577.888672</v>
+      </c>
+      <c r="O35">
+        <v>6614.6298829999996</v>
+      </c>
+      <c r="P35">
+        <v>6684.3378910000001</v>
+      </c>
+      <c r="Q35">
+        <v>6740.0898440000001</v>
+      </c>
+      <c r="R35">
+        <v>6793.6845700000003</v>
+      </c>
+      <c r="S35">
+        <v>6856.6494140000004</v>
+      </c>
+      <c r="T35">
+        <v>6918.3007809999999</v>
+      </c>
+      <c r="U35">
+        <v>6987.3964839999999</v>
+      </c>
+      <c r="V35">
+        <v>7063.0190430000002</v>
+      </c>
+      <c r="W35">
+        <v>7128.4624020000001</v>
+      </c>
+      <c r="X35">
+        <v>7196.8632809999999</v>
+      </c>
+      <c r="Y35">
+        <v>7256.607422</v>
+      </c>
+      <c r="Z35">
+        <v>7322.8701170000004</v>
+      </c>
+      <c r="AA35">
+        <v>7384.330078</v>
+      </c>
+      <c r="AB35">
+        <v>7454.5502930000002</v>
+      </c>
+      <c r="AC35">
+        <v>7535.2553710000002</v>
+      </c>
+      <c r="AD35">
+        <v>7606.2373049999997</v>
+      </c>
+      <c r="AE35">
+        <v>7681.5273440000001</v>
+      </c>
+      <c r="AF35">
+        <v>7743.6040039999998</v>
+      </c>
+      <c r="AG35" s="38">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" t="s">
+        <v>185</v>
+      </c>
+      <c r="C36" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36" t="s">
+        <v>178</v>
+      </c>
+      <c r="F36">
+        <v>2316.6770019999999</v>
+      </c>
+      <c r="G36">
+        <v>2344.0678710000002</v>
+      </c>
+      <c r="H36">
+        <v>2344.7004390000002</v>
+      </c>
+      <c r="I36">
+        <v>2344.4560550000001</v>
+      </c>
+      <c r="J36">
+        <v>2339.9897460000002</v>
+      </c>
+      <c r="K36">
+        <v>2341.404297</v>
+      </c>
+      <c r="L36">
+        <v>2345.9621579999998</v>
+      </c>
+      <c r="M36">
+        <v>2352.5458979999999</v>
+      </c>
+      <c r="N36">
+        <v>2357.4746089999999</v>
+      </c>
+      <c r="O36">
+        <v>2357.0366210000002</v>
+      </c>
+      <c r="P36">
+        <v>2364.6447750000002</v>
+      </c>
+      <c r="Q36">
+        <v>2371.5659179999998</v>
+      </c>
+      <c r="R36">
+        <v>2377.9558109999998</v>
+      </c>
+      <c r="S36">
+        <v>2386.4594729999999</v>
+      </c>
+      <c r="T36">
+        <v>2396.358154</v>
+      </c>
+      <c r="U36">
+        <v>2410.375</v>
+      </c>
+      <c r="V36">
+        <v>2428.2468260000001</v>
+      </c>
+      <c r="W36">
+        <v>2443.2141109999998</v>
+      </c>
+      <c r="X36">
+        <v>2458.0295409999999</v>
+      </c>
+      <c r="Y36">
+        <v>2472.5490719999998</v>
+      </c>
+      <c r="Z36">
+        <v>2488.7951659999999</v>
+      </c>
+      <c r="AA36">
+        <v>2501.2651369999999</v>
+      </c>
+      <c r="AB36">
+        <v>2515.9790039999998</v>
+      </c>
+      <c r="AC36">
+        <v>2536.919922</v>
+      </c>
+      <c r="AD36">
+        <v>2552.499268</v>
+      </c>
+      <c r="AE36">
+        <v>2569.5615229999999</v>
+      </c>
+      <c r="AF36">
+        <v>2586.6147460000002</v>
+      </c>
+      <c r="AG36" s="38">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B37" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" t="s">
+        <v>181</v>
+      </c>
+      <c r="D37" t="s">
+        <v>178</v>
+      </c>
+      <c r="F37">
+        <v>3658.2871089999999</v>
+      </c>
+      <c r="G37">
+        <v>3758.0356449999999</v>
+      </c>
+      <c r="H37">
+        <v>3875.6811520000001</v>
+      </c>
+      <c r="I37">
+        <v>3953.2326659999999</v>
+      </c>
+      <c r="J37">
+        <v>4019.1171880000002</v>
+      </c>
+      <c r="K37">
+        <v>4078.3217770000001</v>
+      </c>
+      <c r="L37">
+        <v>4133.3310549999997</v>
+      </c>
+      <c r="M37">
+        <v>4171.4423829999996</v>
+      </c>
+      <c r="N37">
+        <v>4220.4150390000004</v>
+      </c>
+      <c r="O37">
+        <v>4257.59375</v>
+      </c>
+      <c r="P37">
+        <v>4319.6933589999999</v>
+      </c>
+      <c r="Q37">
+        <v>4368.5234380000002</v>
+      </c>
+      <c r="R37">
+        <v>4415.7285160000001</v>
+      </c>
+      <c r="S37">
+        <v>4470.1904299999997</v>
+      </c>
+      <c r="T37">
+        <v>4521.9423829999996</v>
+      </c>
+      <c r="U37">
+        <v>4577.0209960000002</v>
+      </c>
+      <c r="V37">
+        <v>4634.7724609999996</v>
+      </c>
+      <c r="W37">
+        <v>4685.2485349999997</v>
+      </c>
+      <c r="X37">
+        <v>4738.8339839999999</v>
+      </c>
+      <c r="Y37">
+        <v>4784.0585940000001</v>
+      </c>
+      <c r="Z37">
+        <v>4834.0747069999998</v>
+      </c>
+      <c r="AA37">
+        <v>4883.0659180000002</v>
+      </c>
+      <c r="AB37">
+        <v>4938.5712890000004</v>
+      </c>
+      <c r="AC37">
+        <v>4998.3364259999998</v>
+      </c>
+      <c r="AD37">
+        <v>5053.7377930000002</v>
+      </c>
+      <c r="AE37">
+        <v>5111.9658200000003</v>
+      </c>
+      <c r="AF37">
+        <v>5156.9897460000002</v>
+      </c>
+      <c r="AG37" s="38">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>81</v>
+      </c>
+      <c r="B38" t="s">
+        <v>180</v>
+      </c>
+      <c r="C38" t="s">
+        <v>179</v>
+      </c>
+      <c r="D38" t="s">
+        <v>178</v>
+      </c>
+      <c r="F38">
+        <v>36919.445312000003</v>
+      </c>
+      <c r="G38">
+        <v>37712.523437999997</v>
+      </c>
+      <c r="H38">
+        <v>38555.71875</v>
+      </c>
+      <c r="I38">
+        <v>39495.554687999997</v>
+      </c>
+      <c r="J38">
+        <v>40443.34375</v>
+      </c>
+      <c r="K38">
+        <v>41284.398437999997</v>
+      </c>
+      <c r="L38">
+        <v>42024.367187999997</v>
+      </c>
+      <c r="M38">
+        <v>42737.675780999998</v>
+      </c>
+      <c r="N38">
+        <v>43501.859375</v>
+      </c>
+      <c r="O38">
+        <v>44242.21875</v>
+      </c>
+      <c r="P38">
+        <v>45019.085937999997</v>
+      </c>
+      <c r="Q38">
+        <v>45789.011719000002</v>
+      </c>
+      <c r="R38">
+        <v>46539.425780999998</v>
+      </c>
+      <c r="S38">
+        <v>47291.625</v>
+      </c>
+      <c r="T38">
+        <v>48035.277344000002</v>
+      </c>
+      <c r="U38">
+        <v>48786.238280999998</v>
+      </c>
+      <c r="V38">
+        <v>49568.90625</v>
+      </c>
+      <c r="W38">
+        <v>50337.425780999998</v>
+      </c>
+      <c r="X38">
+        <v>51120.59375</v>
+      </c>
+      <c r="Y38">
+        <v>51888.730469000002</v>
+      </c>
+      <c r="Z38">
+        <v>52670.605469000002</v>
+      </c>
+      <c r="AA38">
+        <v>53466.746094000002</v>
+      </c>
+      <c r="AB38">
+        <v>54291.320312000003</v>
+      </c>
+      <c r="AC38">
+        <v>55161.792969000002</v>
+      </c>
+      <c r="AD38">
+        <v>56045.03125</v>
+      </c>
+      <c r="AE38">
+        <v>56967.78125</v>
+      </c>
+      <c r="AF38">
+        <v>57872.921875</v>
+      </c>
+      <c r="AG38" s="38">
+        <v>1.7000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>171</v>
+      </c>
+      <c r="B40" t="s">
+        <v>177</v>
+      </c>
+      <c r="C40" t="s">
+        <v>176</v>
+      </c>
+      <c r="D40" t="s">
+        <v>175</v>
+      </c>
+      <c r="E40" t="s">
+        <v>135</v>
+      </c>
+      <c r="G40">
+        <v>342.00198399999999</v>
+      </c>
+      <c r="H40">
+        <v>344.85076900000001</v>
+      </c>
+      <c r="I40">
+        <v>346.96423299999998</v>
+      </c>
+      <c r="J40">
+        <v>348.437408</v>
+      </c>
+      <c r="K40">
+        <v>349.87805200000003</v>
+      </c>
+      <c r="L40">
+        <v>351.28118899999998</v>
+      </c>
+      <c r="M40">
+        <v>352.64178500000003</v>
+      </c>
+      <c r="N40">
+        <v>353.95739700000001</v>
+      </c>
+      <c r="O40">
+        <v>355.23046900000003</v>
+      </c>
+      <c r="P40">
+        <v>356.458527</v>
+      </c>
+      <c r="Q40">
+        <v>357.63406400000002</v>
+      </c>
+      <c r="R40">
+        <v>358.73593099999999</v>
+      </c>
+      <c r="S40">
+        <v>359.77282700000001</v>
+      </c>
+      <c r="T40">
+        <v>360.75125100000002</v>
+      </c>
+      <c r="U40">
+        <v>361.67263800000001</v>
+      </c>
+      <c r="V40">
+        <v>362.53564499999999</v>
+      </c>
+      <c r="W40">
+        <v>363.34353599999997</v>
+      </c>
+      <c r="X40">
+        <v>364.09573399999999</v>
+      </c>
+      <c r="Y40">
+        <v>364.79132099999998</v>
+      </c>
+      <c r="Z40">
+        <v>365.436127</v>
+      </c>
+      <c r="AA40">
+        <v>366.03445399999998</v>
+      </c>
+      <c r="AB40">
+        <v>366.59066799999999</v>
+      </c>
+      <c r="AC40">
+        <v>367.10647599999999</v>
+      </c>
+      <c r="AD40">
+        <v>367.58792099999999</v>
+      </c>
+      <c r="AE40">
+        <v>368.03945900000002</v>
+      </c>
+      <c r="AF40">
+        <v>368.46582000000001</v>
+      </c>
+      <c r="AG40">
+        <v>368.87057499999997</v>
+      </c>
+      <c r="AH40" s="38">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>171</v>
+      </c>
+      <c r="B41" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" t="s">
+        <v>173</v>
+      </c>
+      <c r="D41" t="s">
+        <v>172</v>
+      </c>
+      <c r="E41" t="s">
+        <v>135</v>
+      </c>
+      <c r="G41">
+        <v>277.99807700000002</v>
+      </c>
+      <c r="H41">
+        <v>280.90438799999998</v>
+      </c>
+      <c r="I41">
+        <v>283.17041</v>
+      </c>
+      <c r="J41">
+        <v>284.87118500000003</v>
+      </c>
+      <c r="K41">
+        <v>286.50192299999998</v>
+      </c>
+      <c r="L41">
+        <v>288.10513300000002</v>
+      </c>
+      <c r="M41">
+        <v>289.69085699999999</v>
+      </c>
+      <c r="N41">
+        <v>291.249054</v>
+      </c>
+      <c r="O41">
+        <v>292.72473100000002</v>
+      </c>
+      <c r="P41">
+        <v>294.080353</v>
+      </c>
+      <c r="Q41">
+        <v>295.31839000000002</v>
+      </c>
+      <c r="R41">
+        <v>296.44641100000001</v>
+      </c>
+      <c r="S41">
+        <v>297.47686800000002</v>
+      </c>
+      <c r="T41">
+        <v>298.40228300000001</v>
+      </c>
+      <c r="U41">
+        <v>299.38275099999998</v>
+      </c>
+      <c r="V41">
+        <v>300.31817599999999</v>
+      </c>
+      <c r="W41">
+        <v>301.21105999999997</v>
+      </c>
+      <c r="X41">
+        <v>302.063965</v>
+      </c>
+      <c r="Y41">
+        <v>302.88681000000003</v>
+      </c>
+      <c r="Z41">
+        <v>303.67718500000001</v>
+      </c>
+      <c r="AA41">
+        <v>304.44003300000003</v>
+      </c>
+      <c r="AB41">
+        <v>305.17785600000002</v>
+      </c>
+      <c r="AC41">
+        <v>305.89819299999999</v>
+      </c>
+      <c r="AD41">
+        <v>306.60101300000002</v>
+      </c>
+      <c r="AE41">
+        <v>307.29382299999997</v>
+      </c>
+      <c r="AF41">
+        <v>307.96661399999999</v>
+      </c>
+      <c r="AG41">
+        <v>308.62692299999998</v>
+      </c>
+      <c r="AH41" s="38">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>171</v>
+      </c>
+      <c r="B42" t="s">
+        <v>170</v>
+      </c>
+      <c r="C42" t="s">
+        <v>169</v>
+      </c>
+      <c r="D42" t="s">
+        <v>168</v>
+      </c>
+      <c r="E42" t="s">
+        <v>135</v>
+      </c>
+      <c r="G42">
+        <v>61.577815999999999</v>
+      </c>
+      <c r="H42">
+        <v>63.338611999999998</v>
+      </c>
+      <c r="I42">
+        <v>65.071892000000005</v>
+      </c>
+      <c r="J42">
+        <v>66.737647999999993</v>
+      </c>
+      <c r="K42">
+        <v>68.305854999999994</v>
+      </c>
+      <c r="L42">
+        <v>69.771514999999994</v>
+      </c>
+      <c r="M42">
+        <v>71.052093999999997</v>
+      </c>
+      <c r="N42">
+        <v>72.125084000000001</v>
+      </c>
+      <c r="O42">
+        <v>73.070510999999996</v>
+      </c>
+      <c r="P42">
+        <v>73.940903000000006</v>
+      </c>
+      <c r="Q42">
+        <v>74.821297000000001</v>
+      </c>
+      <c r="R42">
+        <v>75.754219000000006</v>
+      </c>
+      <c r="S42">
+        <v>76.622107999999997</v>
+      </c>
+      <c r="T42">
+        <v>77.209877000000006</v>
+      </c>
+      <c r="U42">
+        <v>77.577545000000001</v>
+      </c>
+      <c r="V42">
+        <v>77.862671000000006</v>
+      </c>
+      <c r="W42">
+        <v>78.140297000000004</v>
+      </c>
+      <c r="X42">
+        <v>78.365402000000003</v>
+      </c>
+      <c r="Y42">
+        <v>78.663032999999999</v>
+      </c>
+      <c r="Z42">
+        <v>78.975677000000005</v>
+      </c>
+      <c r="AA42">
+        <v>79.355850000000004</v>
+      </c>
+      <c r="AB42">
+        <v>79.833564999999993</v>
+      </c>
+      <c r="AC42">
+        <v>80.308777000000006</v>
+      </c>
+      <c r="AD42">
+        <v>80.819007999999997</v>
+      </c>
+      <c r="AE42">
+        <v>81.304230000000004</v>
+      </c>
+      <c r="AF42">
+        <v>81.759429999999995</v>
+      </c>
+      <c r="AG42">
+        <v>82.294678000000005</v>
+      </c>
+      <c r="AH42" s="38">
+        <v>1.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>164</v>
+      </c>
+      <c r="B43" t="s">
+        <v>167</v>
+      </c>
+      <c r="C43" t="s">
+        <v>166</v>
+      </c>
+      <c r="D43" t="s">
+        <v>165</v>
+      </c>
+      <c r="E43" t="s">
+        <v>135</v>
+      </c>
+      <c r="G43">
+        <v>159.54521199999999</v>
+      </c>
+      <c r="H43">
+        <v>160.89846800000001</v>
+      </c>
+      <c r="I43">
+        <v>161.43066400000001</v>
+      </c>
+      <c r="J43">
+        <v>161.697113</v>
+      </c>
+      <c r="K43">
+        <v>161.99790999999999</v>
+      </c>
+      <c r="L43">
+        <v>162.53140300000001</v>
+      </c>
+      <c r="M43">
+        <v>163.241547</v>
+      </c>
+      <c r="N43">
+        <v>163.92671200000001</v>
+      </c>
+      <c r="O43">
+        <v>164.54892000000001</v>
+      </c>
+      <c r="P43">
+        <v>164.98477199999999</v>
+      </c>
+      <c r="Q43">
+        <v>165.29776000000001</v>
+      </c>
+      <c r="R43">
+        <v>165.56591800000001</v>
+      </c>
+      <c r="S43">
+        <v>166.08338900000001</v>
+      </c>
+      <c r="T43">
+        <v>166.79139699999999</v>
+      </c>
+      <c r="U43">
+        <v>167.53140300000001</v>
+      </c>
+      <c r="V43">
+        <v>168.18656899999999</v>
+      </c>
+      <c r="W43">
+        <v>169.00384500000001</v>
+      </c>
+      <c r="X43">
+        <v>169.658646</v>
+      </c>
+      <c r="Y43">
+        <v>170.29731799999999</v>
+      </c>
+      <c r="Z43">
+        <v>170.74044799999999</v>
+      </c>
+      <c r="AA43">
+        <v>171.20611600000001</v>
+      </c>
+      <c r="AB43">
+        <v>171.654968</v>
+      </c>
+      <c r="AC43">
+        <v>172.127533</v>
+      </c>
+      <c r="AD43">
+        <v>172.64163199999999</v>
+      </c>
+      <c r="AE43">
+        <v>173.163284</v>
+      </c>
+      <c r="AF43">
+        <v>173.71743799999999</v>
+      </c>
+      <c r="AG43">
+        <v>174.28782699999999</v>
+      </c>
+      <c r="AH43" s="38">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>164</v>
+      </c>
+      <c r="B44" t="s">
+        <v>163</v>
+      </c>
+      <c r="C44" t="s">
+        <v>162</v>
+      </c>
+      <c r="D44" t="s">
+        <v>161</v>
+      </c>
+      <c r="E44" t="s">
+        <v>135</v>
+      </c>
+      <c r="G44">
+        <v>12.946291</v>
+      </c>
+      <c r="H44">
+        <v>12.607818</v>
+      </c>
+      <c r="I44">
+        <v>12.266394999999999</v>
+      </c>
+      <c r="J44">
+        <v>12.145358999999999</v>
+      </c>
+      <c r="K44">
+        <v>11.975657</v>
+      </c>
+      <c r="L44">
+        <v>11.855324</v>
+      </c>
+      <c r="M44">
+        <v>11.823164</v>
+      </c>
+      <c r="N44">
+        <v>11.811355000000001</v>
+      </c>
+      <c r="O44">
+        <v>11.753557000000001</v>
+      </c>
+      <c r="P44">
+        <v>11.639316000000001</v>
+      </c>
+      <c r="Q44">
+        <v>11.500506</v>
+      </c>
+      <c r="R44">
+        <v>11.483269</v>
+      </c>
+      <c r="S44">
+        <v>11.548651</v>
+      </c>
+      <c r="T44">
+        <v>11.638992</v>
+      </c>
+      <c r="U44">
+        <v>11.723704</v>
+      </c>
+      <c r="V44">
+        <v>11.786910000000001</v>
+      </c>
+      <c r="W44">
+        <v>11.825393999999999</v>
+      </c>
+      <c r="X44">
+        <v>11.847021</v>
+      </c>
+      <c r="Y44">
+        <v>11.844115</v>
+      </c>
+      <c r="Z44">
+        <v>11.812518000000001</v>
+      </c>
+      <c r="AA44">
+        <v>11.792035</v>
+      </c>
+      <c r="AB44">
+        <v>11.817151000000001</v>
+      </c>
+      <c r="AC44">
+        <v>11.839629</v>
+      </c>
+      <c r="AD44">
+        <v>11.86697</v>
+      </c>
+      <c r="AE44">
+        <v>11.895567</v>
+      </c>
+      <c r="AF44">
+        <v>11.917655999999999</v>
+      </c>
+      <c r="AG44">
+        <v>11.917175</v>
+      </c>
+      <c r="AH44" s="38">
+        <v>-3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>160</v>
+      </c>
+      <c r="B46" t="s">
+        <v>159</v>
+      </c>
+      <c r="C46" t="s">
+        <v>158</v>
+      </c>
+      <c r="D46" t="s">
+        <v>135</v>
+      </c>
+      <c r="F46">
+        <v>168.244507</v>
+      </c>
+      <c r="G46">
+        <v>169.61247299999999</v>
+      </c>
+      <c r="H46">
+        <v>170.370926</v>
+      </c>
+      <c r="I46">
+        <v>170.93872099999999</v>
+      </c>
+      <c r="J46">
+        <v>171.43718000000001</v>
+      </c>
+      <c r="K46">
+        <v>171.976822</v>
+      </c>
+      <c r="L46">
+        <v>172.528076</v>
+      </c>
+      <c r="M46">
+        <v>172.99882500000001</v>
+      </c>
+      <c r="N46">
+        <v>173.50010700000001</v>
+      </c>
+      <c r="O46">
+        <v>173.97044399999999</v>
+      </c>
+      <c r="P46">
+        <v>174.39047199999999</v>
+      </c>
+      <c r="Q46">
+        <v>174.836533</v>
+      </c>
+      <c r="R46">
+        <v>175.40377799999999</v>
+      </c>
+      <c r="S46">
+        <v>176.1875</v>
+      </c>
+      <c r="T46">
+        <v>177.08592200000001</v>
+      </c>
+      <c r="U46">
+        <v>177.926468</v>
+      </c>
+      <c r="V46">
+        <v>178.68949900000001</v>
+      </c>
+      <c r="W46">
+        <v>179.39688100000001</v>
+      </c>
+      <c r="X46">
+        <v>179.99130199999999</v>
+      </c>
+      <c r="Y46">
+        <v>180.49859599999999</v>
+      </c>
+      <c r="Z46">
+        <v>180.95825199999999</v>
+      </c>
+      <c r="AA46">
+        <v>181.417801</v>
+      </c>
+      <c r="AB46">
+        <v>181.86991900000001</v>
+      </c>
+      <c r="AC46">
+        <v>182.33622700000001</v>
+      </c>
+      <c r="AD46">
+        <v>182.85797099999999</v>
+      </c>
+      <c r="AE46">
+        <v>183.42129499999999</v>
+      </c>
+      <c r="AF46">
+        <v>183.963303</v>
+      </c>
+      <c r="AG46" s="38">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>157</v>
+      </c>
+      <c r="B47" t="s">
+        <v>156</v>
+      </c>
+      <c r="C47" t="s">
+        <v>155</v>
+      </c>
+      <c r="D47" t="s">
+        <v>154</v>
+      </c>
+      <c r="F47">
+        <v>1.200237</v>
+      </c>
+      <c r="G47">
+        <v>1.2221420000000001</v>
+      </c>
+      <c r="H47">
+        <v>1.2499739999999999</v>
+      </c>
+      <c r="I47">
+        <v>1.2750520000000001</v>
+      </c>
+      <c r="J47">
+        <v>1.2965279999999999</v>
+      </c>
+      <c r="K47">
+        <v>1.3171600000000001</v>
+      </c>
+      <c r="L47">
+        <v>1.335774</v>
+      </c>
+      <c r="M47">
+        <v>1.353707</v>
+      </c>
+      <c r="N47">
+        <v>1.3744730000000001</v>
+      </c>
+      <c r="O47">
+        <v>1.396873</v>
+      </c>
+      <c r="P47">
+        <v>1.4208719999999999</v>
+      </c>
+      <c r="Q47">
+        <v>1.445487</v>
+      </c>
+      <c r="R47">
+        <v>1.469641</v>
+      </c>
+      <c r="S47">
+        <v>1.4949570000000001</v>
+      </c>
+      <c r="T47">
+        <v>1.52258</v>
+      </c>
+      <c r="U47">
+        <v>1.5537099999999999</v>
+      </c>
+      <c r="V47">
+        <v>1.5864050000000001</v>
+      </c>
+      <c r="W47">
+        <v>1.621016</v>
+      </c>
+      <c r="X47">
+        <v>1.6581669999999999</v>
+      </c>
+      <c r="Y47">
+        <v>1.6965870000000001</v>
+      </c>
+      <c r="Z47">
+        <v>1.735201</v>
+      </c>
+      <c r="AA47">
+        <v>1.773522</v>
+      </c>
+      <c r="AB47">
+        <v>1.8128439999999999</v>
+      </c>
+      <c r="AC47">
+        <v>1.852177</v>
+      </c>
+      <c r="AD47">
+        <v>1.8924609999999999</v>
+      </c>
+      <c r="AE47">
+        <v>1.9334450000000001</v>
+      </c>
+      <c r="AF47">
+        <v>1.975163</v>
+      </c>
+      <c r="AG47" s="38">
+        <v>1.9E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>153</v>
+      </c>
+      <c r="B48" t="s">
+        <v>152</v>
+      </c>
+      <c r="C48" t="s">
+        <v>151</v>
+      </c>
+      <c r="D48" t="s">
+        <v>150</v>
+      </c>
+      <c r="F48">
+        <v>4.027698</v>
+      </c>
+      <c r="G48">
+        <v>4.3234389999999996</v>
+      </c>
+      <c r="H48">
+        <v>4.4824020000000004</v>
+      </c>
+      <c r="I48">
+        <v>4.5178050000000001</v>
+      </c>
+      <c r="J48">
+        <v>4.4896529999999997</v>
+      </c>
+      <c r="K48">
+        <v>4.3921130000000002</v>
+      </c>
+      <c r="L48">
+        <v>4.2577109999999996</v>
+      </c>
+      <c r="M48">
+        <v>4.1460800000000004</v>
+      </c>
+      <c r="N48">
+        <v>4.0749360000000001</v>
+      </c>
+      <c r="O48">
+        <v>4.0667340000000003</v>
+      </c>
+      <c r="P48">
+        <v>4.0972730000000004</v>
+      </c>
+      <c r="Q48">
+        <v>4.0881470000000002</v>
+      </c>
+      <c r="R48">
+        <v>4.0768959999999996</v>
+      </c>
+      <c r="S48">
+        <v>4.0943290000000001</v>
+      </c>
+      <c r="T48">
+        <v>4.1547429999999999</v>
+      </c>
+      <c r="U48">
+        <v>4.2350209999999997</v>
+      </c>
+      <c r="V48">
+        <v>4.2689370000000002</v>
+      </c>
+      <c r="W48">
+        <v>4.296646</v>
+      </c>
+      <c r="X48">
+        <v>4.2949960000000003</v>
+      </c>
+      <c r="Y48">
+        <v>4.2819649999999996</v>
+      </c>
+      <c r="Z48">
+        <v>4.2713929999999998</v>
+      </c>
+      <c r="AA48">
+        <v>4.2865690000000001</v>
+      </c>
+      <c r="AB48">
+        <v>4.2942280000000004</v>
+      </c>
+      <c r="AC48">
+        <v>4.2851749999999997</v>
+      </c>
+      <c r="AD48">
+        <v>4.276694</v>
+      </c>
+      <c r="AE48">
+        <v>4.269107</v>
+      </c>
+      <c r="AF48">
+        <v>4.278886</v>
+      </c>
+      <c r="AG48" s="38">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>149</v>
+      </c>
+      <c r="B50" t="s">
+        <v>148</v>
+      </c>
+      <c r="C50" t="s">
+        <v>147</v>
+      </c>
+      <c r="D50" t="s">
+        <v>146</v>
+      </c>
+      <c r="F50">
+        <v>16628.990234000001</v>
+      </c>
+      <c r="G50">
+        <v>17088.570312</v>
+      </c>
+      <c r="H50">
+        <v>17659.257812</v>
+      </c>
+      <c r="I50">
+        <v>18160.914062</v>
+      </c>
+      <c r="J50">
+        <v>18622.626952999999</v>
+      </c>
+      <c r="K50">
+        <v>19065.867188</v>
+      </c>
+      <c r="L50">
+        <v>19500.0625</v>
+      </c>
+      <c r="M50">
+        <v>19916.849609000001</v>
+      </c>
+      <c r="N50">
+        <v>20345.167968999998</v>
+      </c>
+      <c r="O50">
+        <v>20778.535156000002</v>
+      </c>
+      <c r="P50">
+        <v>21232.025390999999</v>
+      </c>
+      <c r="Q50">
+        <v>21663.232422000001</v>
+      </c>
+      <c r="R50">
+        <v>22105.75</v>
+      </c>
+      <c r="S50">
+        <v>22560.574218999998</v>
+      </c>
+      <c r="T50">
+        <v>23022.482422000001</v>
+      </c>
+      <c r="U50">
+        <v>23508.675781000002</v>
+      </c>
+      <c r="V50">
+        <v>24013.269531000002</v>
+      </c>
+      <c r="W50">
+        <v>24495.851562</v>
+      </c>
+      <c r="X50">
+        <v>25000.126952999999</v>
+      </c>
+      <c r="Y50">
+        <v>25509.75</v>
+      </c>
+      <c r="Z50">
+        <v>26027.070312</v>
+      </c>
+      <c r="AA50">
+        <v>26546.287109000001</v>
+      </c>
+      <c r="AB50">
+        <v>27081.972656000002</v>
+      </c>
+      <c r="AC50">
+        <v>27627.421875</v>
+      </c>
+      <c r="AD50">
+        <v>28177.890625</v>
+      </c>
+      <c r="AE50">
+        <v>28739.75</v>
+      </c>
+      <c r="AF50">
+        <v>29311.912109000001</v>
+      </c>
+      <c r="AG50" s="38">
+        <v>2.1999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>145</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51" t="s">
+        <v>135</v>
+      </c>
+      <c r="F51">
+        <v>1.4524600000000001</v>
+      </c>
+      <c r="G51">
+        <v>1.485654</v>
+      </c>
+      <c r="H51">
+        <v>1.5696749999999999</v>
+      </c>
+      <c r="I51">
+        <v>1.5868390000000001</v>
+      </c>
+      <c r="J51">
+        <v>1.5930960000000001</v>
+      </c>
+      <c r="K51">
+        <v>1.6307100000000001</v>
+      </c>
+      <c r="L51">
+        <v>1.630992</v>
+      </c>
+      <c r="M51">
+        <v>1.6331310000000001</v>
+      </c>
+      <c r="N51">
+        <v>1.6178619999999999</v>
+      </c>
+      <c r="O51">
+        <v>1.565299</v>
+      </c>
+      <c r="P51">
+        <v>1.500715</v>
+      </c>
+      <c r="Q51">
+        <v>1.478613</v>
+      </c>
+      <c r="R51">
+        <v>1.4490959999999999</v>
+      </c>
+      <c r="S51">
+        <v>1.392733</v>
+      </c>
+      <c r="T51">
+        <v>1.3415280000000001</v>
+      </c>
+      <c r="U51">
+        <v>1.285423</v>
+      </c>
+      <c r="V51">
+        <v>1.2426429999999999</v>
+      </c>
+      <c r="W51">
+        <v>1.1913050000000001</v>
+      </c>
+      <c r="X51">
+        <v>1.153365</v>
+      </c>
+      <c r="Y51">
+        <v>1.113051</v>
+      </c>
+      <c r="Z51">
+        <v>1.094303</v>
+      </c>
+      <c r="AA51">
+        <v>1.0945009999999999</v>
+      </c>
+      <c r="AB51">
+        <v>1.0915790000000001</v>
+      </c>
+      <c r="AC51">
+        <v>1.0903320000000001</v>
+      </c>
+      <c r="AD51">
+        <v>1.089172</v>
+      </c>
+      <c r="AE51">
+        <v>1.089164</v>
+      </c>
+      <c r="AF51">
+        <v>1.0858350000000001</v>
+      </c>
+      <c r="AG51" s="38">
+        <v>-1.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>142</v>
+      </c>
+      <c r="B52" t="s">
+        <v>141</v>
+      </c>
+      <c r="C52" t="s">
+        <v>140</v>
+      </c>
+      <c r="D52" t="s">
+        <v>139</v>
+      </c>
+      <c r="F52">
+        <v>103.371872</v>
+      </c>
+      <c r="G52">
+        <v>104.52195</v>
+      </c>
+      <c r="H52">
+        <v>105.93501999999999</v>
+      </c>
+      <c r="I52">
+        <v>107.51918000000001</v>
+      </c>
+      <c r="J52">
+        <v>109.194839</v>
+      </c>
+      <c r="K52">
+        <v>110.865685</v>
+      </c>
+      <c r="L52">
+        <v>112.493584</v>
+      </c>
+      <c r="M52">
+        <v>114.092934</v>
+      </c>
+      <c r="N52">
+        <v>115.698303</v>
+      </c>
+      <c r="O52">
+        <v>117.31967899999999</v>
+      </c>
+      <c r="P52">
+        <v>118.94864699999999</v>
+      </c>
+      <c r="Q52">
+        <v>120.570572</v>
+      </c>
+      <c r="R52">
+        <v>122.16892199999999</v>
+      </c>
+      <c r="S52">
+        <v>123.73555</v>
+      </c>
+      <c r="T52">
+        <v>125.27293400000001</v>
+      </c>
+      <c r="U52">
+        <v>126.786034</v>
+      </c>
+      <c r="V52">
+        <v>128.28021200000001</v>
+      </c>
+      <c r="W52">
+        <v>129.76083399999999</v>
+      </c>
+      <c r="X52">
+        <v>131.231323</v>
+      </c>
+      <c r="Y52">
+        <v>132.69490099999999</v>
+      </c>
+      <c r="Z52">
+        <v>134.15536499999999</v>
+      </c>
+      <c r="AA52">
+        <v>135.616333</v>
+      </c>
+      <c r="AB52">
+        <v>137.08107000000001</v>
+      </c>
+      <c r="AC52">
+        <v>138.55230700000001</v>
+      </c>
+      <c r="AD52">
+        <v>140.03160099999999</v>
+      </c>
+      <c r="AE52">
+        <v>141.51960800000001</v>
+      </c>
+      <c r="AF52">
+        <v>143.01623499999999</v>
+      </c>
+      <c r="AG52" s="38">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>138</v>
+      </c>
+      <c r="B53" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" t="s">
+        <v>136</v>
+      </c>
+      <c r="D53" t="s">
+        <v>135</v>
+      </c>
+      <c r="F53">
+        <v>15.735111</v>
+      </c>
+      <c r="G53">
+        <v>16.256453</v>
+      </c>
+      <c r="H53">
+        <v>16.903842999999998</v>
+      </c>
+      <c r="I53">
+        <v>17.003399000000002</v>
+      </c>
+      <c r="J53">
+        <v>16.499796</v>
+      </c>
+      <c r="K53">
+        <v>16.222467000000002</v>
+      </c>
+      <c r="L53">
+        <v>16.024592999999999</v>
+      </c>
+      <c r="M53">
+        <v>15.67191</v>
+      </c>
+      <c r="N53">
+        <v>15.482900000000001</v>
+      </c>
+      <c r="O53">
+        <v>15.518478999999999</v>
+      </c>
+      <c r="P53">
+        <v>15.631788</v>
+      </c>
+      <c r="Q53">
+        <v>15.618696999999999</v>
+      </c>
+      <c r="R53">
+        <v>15.587206</v>
+      </c>
+      <c r="S53">
+        <v>15.601235000000001</v>
+      </c>
+      <c r="T53">
+        <v>15.641641999999999</v>
+      </c>
+      <c r="U53">
+        <v>15.727674</v>
+      </c>
+      <c r="V53">
+        <v>15.74424</v>
+      </c>
+      <c r="W53">
+        <v>15.652267</v>
+      </c>
+      <c r="X53">
+        <v>15.621376</v>
+      </c>
+      <c r="Y53">
+        <v>15.562071</v>
+      </c>
+      <c r="Z53">
+        <v>15.513393000000001</v>
+      </c>
+      <c r="AA53">
+        <v>15.461762999999999</v>
+      </c>
+      <c r="AB53">
+        <v>15.408041000000001</v>
+      </c>
+      <c r="AC53">
+        <v>15.295394</v>
+      </c>
+      <c r="AD53">
+        <v>15.206058000000001</v>
+      </c>
+      <c r="AE53">
+        <v>15.107029000000001</v>
+      </c>
+      <c r="AF53">
+        <v>14.964993</v>
+      </c>
+      <c r="AG53" s="38">
+        <v>-2E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="42"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
@@ -9635,7 +13914,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -9644,7 +13923,7 @@
         <v>19991319900409.637</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -9653,257 +13932,287 @@
         <v>20196793945608.313</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2023</v>
       </c>
       <c r="B4">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A4,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
+        <f>$B$3*INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!A4,'AEO 2023 Table 20'!$13:$13,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
         <v>20353281072644.289</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
       <c r="B5">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A5,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>20549771783508.371</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A5,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>22190278173634.109</v>
+      </c>
+      <c r="F5" s="41"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2025</v>
       </c>
       <c r="B6">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A6,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>20870857005495.758</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A6,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>22673213229081.445</v>
+      </c>
+      <c r="F6" s="41"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
       <c r="B7">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A7,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>21311901045773.098</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A7,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>23198858184475.383</v>
+      </c>
+      <c r="F7" s="41"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2027</v>
       </c>
       <c r="B8">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A8,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>21754391118475.055</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A8,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>23686277139754.777</v>
+      </c>
+      <c r="F8" s="41"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2028</v>
       </c>
       <c r="B9">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A9,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>22171445791271.645</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A9,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>24123360567594.996</v>
+      </c>
+      <c r="F9" s="41"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2029</v>
       </c>
       <c r="B10">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A10,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>22550270469643.211</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A10,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>24586452615706.816</v>
+      </c>
+      <c r="F10" s="41"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2030</v>
       </c>
       <c r="B11">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A11,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>22898069352694.797</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A11,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>25032769482241.699</v>
+      </c>
+      <c r="F11" s="41"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2031</v>
       </c>
       <c r="B12">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A12,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>23256218156822.387</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A12,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>25440402971480.27</v>
+      </c>
+      <c r="F12" s="41"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2032</v>
       </c>
       <c r="B13">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A13,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>23676466485360.797</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A13,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>25871826099382.219</v>
+      </c>
+      <c r="F13" s="41"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2033</v>
       </c>
       <c r="B14">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A14,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>24137525299572.52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A14,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>26313673047194.297</v>
+      </c>
+      <c r="F14" s="41"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2034</v>
       </c>
       <c r="B15">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A15,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>24598983569373.762</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A15,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>26757888772460.664</v>
+      </c>
+      <c r="F15" s="41"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2035</v>
       </c>
       <c r="B16">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A16,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>25065123470669.203</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A16,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>27223727084908.723</v>
+      </c>
+      <c r="F16" s="41"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2036</v>
       </c>
       <c r="B17">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A17,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>25560933012981.219</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A17,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>27690076700797.707</v>
+      </c>
+      <c r="F17" s="41"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2037</v>
       </c>
       <c r="B18">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A18,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>26083606011180.895</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A18,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>28169135029440.816</v>
+      </c>
+      <c r="F18" s="41"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2038</v>
       </c>
       <c r="B19">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A19,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>26620895127074.152</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A19,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>28652183929894.777</v>
+      </c>
+      <c r="F19" s="41"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2039</v>
       </c>
       <c r="B20">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A20,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>27166738606955.355</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A20,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>29147458198812.629</v>
+      </c>
+      <c r="F20" s="41"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2040</v>
       </c>
       <c r="B21">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A21,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>27762753836297.801</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A21,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>29659687404527.227</v>
+      </c>
+      <c r="F21" s="41"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2041</v>
       </c>
       <c r="B22">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A22,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>28361125861185.738</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A22,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>30153587543721.949</v>
+      </c>
+      <c r="F22" s="41"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2042</v>
       </c>
       <c r="B23">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A23,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>28964878565872.152</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A23,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>30669999059398.617</v>
+      </c>
+      <c r="F23" s="41"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2043</v>
       </c>
       <c r="B24">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A24,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>29580740796860.582</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A24,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>31184123687121.258</v>
+      </c>
+      <c r="F24" s="41"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2044</v>
       </c>
       <c r="B25">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A25,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>30194997212779.535</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A25,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>31699131113701.063</v>
+      </c>
+      <c r="F25" s="41"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2045</v>
       </c>
       <c r="B26">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A26,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>30811206972298.781</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A26,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>32214072629045.086</v>
+      </c>
+      <c r="F26" s="41"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2046</v>
       </c>
       <c r="B27">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A27,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>31442737889281.586</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A27,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>32745335943094.758</v>
+      </c>
+      <c r="F27" s="41"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2047</v>
       </c>
       <c r="B28">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A28,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>32098825402645.672</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A28,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>33282351431336.531</v>
+      </c>
+      <c r="F28" s="41"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2048</v>
       </c>
       <c r="B29">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A29,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>32764360063608.441</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A29,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>33822406784140.973</v>
+      </c>
+      <c r="F29" s="41"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2049</v>
       </c>
       <c r="B30">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A30,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>33437811955134.973</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A30,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>34377715388063.188</v>
+      </c>
+      <c r="F30" s="41"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2050</v>
       </c>
       <c r="B31">
-        <f>$B$3*INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!A31,'AEO Table 20'!$13:$13,0))/INDEX('AEO Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO Table 20'!$13:$13,0))</f>
-        <v>34160235230153.73</v>
-      </c>
+        <f>$B$3*INDEX('AEO 2025 Table 20'!$F$6:$AG$6,MATCH(BGDP!A31,'AEO 2025 Table 20'!$F$5:$AG$5,0))/INDEX('AEO 2023 Table 20'!$15:$15,MATCH(BGDP!$A$3,'AEO 2023 Table 20'!$13:$13,0))</f>
+        <v>34935105160678.949</v>
+      </c>
+      <c r="F31" s="41"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D32" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates IO data to newer BEA data and addresses inconsistency with natural gas distribution/pipelines
</commit_message>
<xml_diff>
--- a/InputData/io-model/BGDP/BAU GDP.xlsx
+++ b/InputData/io-model/BGDP/BAU GDP.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\io-model\BGDP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\EPS Structure Research\isic42-staging\io-model\BGDP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FE0D61-2291-4BFC-B39D-37295FF43AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_72C7682CD77EA3C4DCD6D9F52A147D8EBD6A8211" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BEA Data" sheetId="2" r:id="rId2"/>
     <sheet name="AEO 2025 Table 20" sheetId="3" r:id="rId3"/>
-    <sheet name="AEO 2026 Table 20" sheetId="6" r:id="rId4"/>
+    <sheet name="AEO 2026 Table 20" sheetId="4" r:id="rId4"/>
     <sheet name="calcs" sheetId="5" r:id="rId5"/>
-    <sheet name="BGDP" sheetId="4" r:id="rId6"/>
+    <sheet name="BGDP" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -67,12 +67,18 @@
     <t>EIA</t>
   </si>
   <si>
+    <t>Annual Energy Outlook 2026</t>
+  </si>
+  <si>
     <t>https://www.eia.gov/outlooks/aeo/tables_ref.php</t>
   </si>
   <si>
     <t>Table 20</t>
   </si>
   <si>
+    <t>Alternative Electricity and Transportation</t>
+  </si>
+  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -565,247 +571,241 @@
     <t>AEO.2025.HIGHZTC.KEI_SAL_TRN_LDV_NA_NA_NA_MILL.A</t>
   </si>
   <si>
+    <t>https://www.eia.gov/outlooks/aeo/data/browser/#/?id=18-AEO2026&amp;cases=electrnp&amp;sourcekey=0</t>
+  </si>
+  <si>
+    <t>Thu Apr 23 2026 15:00:34 GMT-0700 (Pacific Daylight Time)</t>
+  </si>
+  <si>
+    <t>Growth (2025-2050)</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Real Gross Domestic Product: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_REAL_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Consumption: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RCNSP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Business Fixed Investment: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RINV_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Government Spending: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RGSP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Exports: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_REXP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: GDP Components: Real Imports: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RIMP_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Energy Intensity: Delivered Energy: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.INY_NA_NA_NA_DELE_NA_NA_THBTUPDLRGDP.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Energy Intensity: Total Energy: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.INY_NA_NA_NA_TEN_NA_NA_THBTUPDLRGDP.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Price Indices: GDP Chain-type Price Index: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_GDP_NA_NA_Y09EQ1D3Z.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Consumer Price Index: All-Urban: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_CPI_URB_NA_IDX82TO84EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Consumer Price Index: Energy Commodities and Services: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_CPI_ENE_NA_IDX82TO84EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: All Commodities: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_NA_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Fuel and Power: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_FULP_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Metals and Metal Products: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_MET_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Wholesale Price Index: Industrial Commodities Excluding Energy: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_INDCOM_NA_IDX82EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: Federal Funds Rate: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_FFR_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: 10-Year Treasury Note: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_TNR10_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Interest Rates: AA Utility Bond Rate: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_AAUTR_NA_NA_NA_NA_NA_PCNTN.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Non-Industrial: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_NIND_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Total Industrial: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_IDAL_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Agriculture, Mining, and Construction: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_NMFG_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Manufacturing: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_MANF_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Energy-Intensive: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_EINT_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Non-Energy-Intensive: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_NEINT_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Value of Shipments: Total: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_VOS_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, with Armed Forces Overseas: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.DMG_POP_PWAF_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, aged 16 and over: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.DMG_POP_16+_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Population, aged 65 and over: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.DMG_POP_65+_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Employment, Nonfarm: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.DMG_EMPM_NOFM_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Employment, Manufacturing: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.DMG_EMPM_MANF_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Labor Force: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_LBF_NA_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Nonfarm Labor Productivity: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_LP_NOFM_NA_NA_NA_NA_Y09EQ1.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Labor Indicators: Unemployment Rate: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_UER_NA_NA_NA_NA_NA_PCT.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Real Disposable Personal Income: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_PEI_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Housing Starts: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_HST_NA_NA_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Commercial Floorspace: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.ECI_FLR_COMM_NA_NA_NA_NA_BLNSQFT.A</t>
+  </si>
+  <si>
+    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Unit Sales of Light-Duty Vehicles: Alternative Electricity and Transportation</t>
+  </si>
+  <si>
+    <t>AEO.2026.ELECTRNP.KEI_SAL_TRN_LDV_NA_NA_NA_MILL.A</t>
+  </si>
+  <si>
     <t>Unit: 2012 USD</t>
   </si>
   <si>
-    <t>GDP</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.KEI_SAL_TRN_LDV_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Unit Sales of Light-Duty Vehicles: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_FLR_COMM_NA_NA_NA_NA_BLNSQFT.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Commercial Floorspace: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_HST_NA_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Housing Starts: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_PEI_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Indicators for Energy Use: Real Disposable Personal Income: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_UER_NA_NA_NA_NA_NA_PCT.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Labor Indicators: Unemployment Rate: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_LP_NOFM_NA_NA_NA_NA_Y09EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Labor Indicators: Nonfarm Labor Productivity: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_LBF_NA_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Key Labor Indicators: Labor Force: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.DMG_EMPM_MANF_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Employment, Manufacturing: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.DMG_EMPM_NOFM_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Employment, Nonfarm: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.DMG_POP_65+_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Population, aged 65 and over: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.DMG_POP_16+_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Population, aged 16 and over: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.DMG_POP_PWAF_NA_NA_NA_NA_MILL.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Population, with Armed Forces Overseas: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_NA_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Total: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_NEINT_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Non-Energy-Intensive: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_EINT_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Energy-Intensive: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_MANF_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Manufacturing: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_NMFG_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Agriculture, Mining, and Construction: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_IDAL_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Total Industrial: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_VOS_NIND_NA_NA_NA_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Value of Shipments: Non-Industrial: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_AAUTR_NA_NA_NA_NA_NA_PCNTN.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Interest Rates: AA Utility Bond Rate: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_TNR10_NA_NA_NA_NA_NA_PCNTN.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Interest Rates: 10-Year Treasury Note: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_FFR_NA_NA_NA_NA_NA_PCNTN.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Interest Rates: Federal Funds Rate: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_INDCOM_NA_IDX82EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Wholesale Price Index: Industrial Commodities Excluding Energy: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_MET_NA_IDX82EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Wholesale Price Index: Metals and Metal Products: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_FULP_NA_IDX82EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Wholesale Price Index: Fuel and Power: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_WHP_NA_NA_IDX82EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Wholesale Price Index: All Commodities: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_CPI_ENE_NA_IDX82TO84EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Consumer Price Index: Energy Commodities and Services: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_CPI_URB_NA_IDX82TO84EQ1.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Consumer Price Index: All-Urban: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_INDX_NA_NA_GDP_NA_NA_Y09EQ1D3Z.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Price Indices: GDP Chain-type Price Index: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.INY_NA_NA_NA_TEN_NA_NA_THBTUPDLRGDP.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Energy Intensity: Total Energy: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.INY_NA_NA_NA_DELE_NA_NA_THBTUPDLRGDP.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Energy Intensity: Delivered Energy: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RIMP_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: GDP Components: Real Imports: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_REXP_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: GDP Components: Real Exports: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RGSP_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: GDP Components: Real Government Spending: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RINV_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: GDP Components: Real Business Fixed Investment: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_RCNSP_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: GDP Components: Real Consumption: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>AEO.2026.ELECTRNP.ECI_NA_NA_NA_GDP_REAL_NA_BLNY09DLR.A</t>
-  </si>
-  <si>
-    <t>Macroeconomic Indicators: Real Gross Domestic Product: Alternative Electricity and Transportation</t>
-  </si>
-  <si>
-    <t>Growth (2025-2050)</t>
-  </si>
-  <si>
-    <t>Thu Apr 23 2026 15:00:34 GMT-0700 (Pacific Daylight Time)</t>
-  </si>
-  <si>
-    <t>https://www.eia.gov/outlooks/aeo/data/browser/#/?id=18-AEO2026&amp;cases=electrnp&amp;sourcekey=0</t>
-  </si>
-  <si>
-    <t>Annual Energy Outlook 2026</t>
-  </si>
-  <si>
-    <t>Alternative Electricity and Transportation</t>
+    <t>GDP  {2025+ recomputed: AEO 2026 ELECTRNP real-GDP growth, 2025 spliced vs AEO 2025 (consistent with the Table-23 industrial rates); &lt;=2024 unchanged BEA-anchored history. Scheme-independent: 42-code BGDP == 52-code BGDP (no ISIC dimension).}</t>
   </si>
 </sst>
 </file>
@@ -1355,32 +1355,32 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>254</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>255</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
         <v>0.84730412960844359</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
         <v>0.78452102304761584</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1407,7 +1407,7 @@
         <v>0.75350342301658668</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1415,7 +1415,7 @@
         <v>0.73191600598044548</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1441,43 +1441,43 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" s="10">
         <v>23725645</v>
@@ -1495,7 +1495,7 @@
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="12"/>
       <c r="C5" s="17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5">
         <f t="array" ref="D5:G5">D3:G3*TRANSPOSE(About!A20:A23)</f>
@@ -1526,22 +1526,22 @@
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4">
         <f>G6/F6*'BEA Data'!G5</f>
@@ -1550,13 +1550,13 @@
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5">
         <v>2023</v>
@@ -1643,21 +1643,21 @@
         <v>2050</v>
       </c>
       <c r="AG5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" s="14">
         <v>21699.671875</v>
@@ -1746,21 +1746,21 @@
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
         <v>42</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" t="s">
-        <v>40</v>
       </c>
       <c r="F8">
         <v>15151.048828000001</v>
@@ -1849,16 +1849,16 @@
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F9">
         <v>3493.9401859999998</v>
@@ -1947,16 +1947,16 @@
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F10">
         <v>3663.0996089999999</v>
@@ -2045,16 +2045,16 @@
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F11">
         <v>2721.9965820000002</v>
@@ -2143,16 +2143,16 @@
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F12">
         <v>4085.1303710000002</v>
@@ -2241,26 +2241,26 @@
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F15">
         <v>3.4284460000000001</v>
@@ -2349,16 +2349,16 @@
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" t="s">
         <v>64</v>
-      </c>
-      <c r="C16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" t="s">
-        <v>62</v>
       </c>
       <c r="F16">
         <v>4.3222800000000001</v>
@@ -2447,21 +2447,21 @@
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F18">
         <v>1.3431169999999999</v>
@@ -2550,21 +2550,21 @@
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F20">
         <v>3.1332360000000001</v>
@@ -2653,16 +2653,16 @@
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D21" t="s">
         <v>77</v>
-      </c>
-      <c r="C21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" t="s">
-        <v>75</v>
       </c>
       <c r="F21">
         <v>2.7925080000000002</v>
@@ -2751,21 +2751,21 @@
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F23">
         <v>2.5444830000000001</v>
@@ -2854,16 +2854,16 @@
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" t="s">
         <v>85</v>
-      </c>
-      <c r="C24" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" t="s">
-        <v>83</v>
       </c>
       <c r="F24">
         <v>2.310759</v>
@@ -2952,16 +2952,16 @@
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F25">
         <v>3.0321470000000001</v>
@@ -3050,16 +3050,16 @@
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C26" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F26">
         <v>2.5845829999999999</v>
@@ -3148,24 +3148,24 @@
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F28">
         <v>5.145988</v>
@@ -3254,16 +3254,16 @@
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" t="s">
+        <v>103</v>
+      </c>
+      <c r="D29" t="s">
         <v>100</v>
-      </c>
-      <c r="C29" t="s">
-        <v>101</v>
-      </c>
-      <c r="D29" t="s">
-        <v>98</v>
       </c>
       <c r="F29">
         <v>4.0761909999999997</v>
@@ -3352,16 +3352,16 @@
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F30">
         <v>5.3953499999999996</v>
@@ -3450,21 +3450,21 @@
     </row>
     <row r="31" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F32">
         <v>28226.228515999999</v>
@@ -3553,16 +3553,16 @@
     </row>
     <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B33" t="s">
+        <v>113</v>
+      </c>
+      <c r="C33" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" t="s">
         <v>111</v>
-      </c>
-      <c r="C33" t="s">
-        <v>112</v>
-      </c>
-      <c r="D33" t="s">
-        <v>109</v>
       </c>
       <c r="F33">
         <v>8693.2148440000001</v>
@@ -3651,22 +3651,22 @@
     </row>
     <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F34" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H34">
         <v>2718.2504880000001</v>
@@ -3755,16 +3755,16 @@
     </row>
     <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B35" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F35">
         <v>5974.9643550000001</v>
@@ -3853,16 +3853,16 @@
     </row>
     <row r="36" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C36" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F36">
         <v>2316.6770019999999</v>
@@ -3951,16 +3951,16 @@
     </row>
     <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B37" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D37" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F37">
         <v>3658.2871089999999</v>
@@ -4049,16 +4049,16 @@
     </row>
     <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C38" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F38">
         <v>36919.445312000003</v>
@@ -4147,24 +4147,24 @@
     </row>
     <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B40" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G40">
         <v>342.00198399999999</v>
@@ -4253,19 +4253,19 @@
     </row>
     <row r="41" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
+        <v>139</v>
+      </c>
+      <c r="D41" t="s">
+        <v>140</v>
+      </c>
+      <c r="E41" t="s">
         <v>137</v>
-      </c>
-      <c r="D41" t="s">
-        <v>138</v>
-      </c>
-      <c r="E41" t="s">
-        <v>135</v>
       </c>
       <c r="G41">
         <v>277.99807700000002</v>
@@ -4354,19 +4354,19 @@
     </row>
     <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G42">
         <v>61.577815999999999</v>
@@ -4455,19 +4455,19 @@
     </row>
     <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B43" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C43" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D43" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E43" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G43">
         <v>159.54521199999999</v>
@@ -4556,19 +4556,19 @@
     </row>
     <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C44" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D44" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E44" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G44">
         <v>12.946291</v>
@@ -4657,21 +4657,21 @@
     </row>
     <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B46" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C46" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D46" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F46">
         <v>168.244507</v>
@@ -4760,16 +4760,16 @@
     </row>
     <row r="47" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B47" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C47" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F47">
         <v>1.200237</v>
@@ -4858,16 +4858,16 @@
     </row>
     <row r="48" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B48" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C48" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D48" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F48">
         <v>4.027698</v>
@@ -4956,21 +4956,21 @@
     </row>
     <row r="49" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B50" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C50" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F50">
         <v>16628.990234000001</v>
@@ -5059,16 +5059,16 @@
     </row>
     <row r="51" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B51" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C51" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D51" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F51">
         <v>1.4524600000000001</v>
@@ -5157,16 +5157,16 @@
     </row>
     <row r="52" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B52" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C52" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F52">
         <v>103.371872</v>
@@ -5255,16 +5255,16 @@
     </row>
     <row r="53" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B53" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C53" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F53">
         <v>15.735111</v>
@@ -5357,7 +5357,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A77C9D-436D-4E5A-B1E9-10C612B3587F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AG53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5367,33 +5367,33 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>253</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>252</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5">
         <v>2025</v>
@@ -5474,21 +5474,21 @@
         <v>2050</v>
       </c>
       <c r="AE5" t="s">
-        <v>251</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="C6" t="s">
-        <v>249</v>
+        <v>181</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6">
         <v>22086.083984000001</v>
@@ -5574,21 +5574,21 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D8" t="s">
         <v>42</v>
-      </c>
-      <c r="B8" t="s">
-        <v>248</v>
-      </c>
-      <c r="C8" t="s">
-        <v>247</v>
-      </c>
-      <c r="D8" t="s">
-        <v>40</v>
       </c>
       <c r="E8">
         <v>15470.457031</v>
@@ -5674,16 +5674,16 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>246</v>
+        <v>184</v>
       </c>
       <c r="C9" t="s">
-        <v>245</v>
+        <v>185</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9">
         <v>3563.6354980000001</v>
@@ -5769,16 +5769,16 @@
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>244</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
-        <v>243</v>
+        <v>187</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E10">
         <v>3737.1342770000001</v>
@@ -5864,16 +5864,16 @@
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>242</v>
+        <v>188</v>
       </c>
       <c r="C11" t="s">
-        <v>241</v>
+        <v>189</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E11">
         <v>2741.9916990000002</v>
@@ -5959,16 +5959,16 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C12" t="s">
-        <v>239</v>
+        <v>191</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E12">
         <v>4186.7524409999996</v>
@@ -6054,26 +6054,26 @@
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>238</v>
+        <v>192</v>
       </c>
       <c r="C15" t="s">
-        <v>237</v>
+        <v>193</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E15">
         <v>3.439244</v>
@@ -6159,16 +6159,16 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>236</v>
+        <v>194</v>
       </c>
       <c r="C16" t="s">
-        <v>235</v>
+        <v>195</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16">
         <v>4.314489</v>
@@ -6254,21 +6254,21 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>234</v>
+        <v>196</v>
       </c>
       <c r="C18" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E18">
         <v>1.383637</v>
@@ -6354,21 +6354,21 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
-        <v>231</v>
+        <v>199</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E20">
         <v>3.2241629999999999</v>
@@ -6454,16 +6454,16 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C21" t="s">
-        <v>229</v>
+        <v>201</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E21">
         <v>2.7731669999999999</v>
@@ -6549,21 +6549,21 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>228</v>
+        <v>202</v>
       </c>
       <c r="C23" t="s">
-        <v>227</v>
+        <v>203</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E23">
         <v>2.5913550000000001</v>
@@ -6649,16 +6649,16 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="C24" t="s">
-        <v>225</v>
+        <v>205</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E24">
         <v>2.2429079999999999</v>
@@ -6744,16 +6744,16 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="C25" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E25">
         <v>3.2021440000000001</v>
@@ -6839,16 +6839,16 @@
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B26" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="C26" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E26">
         <v>2.6622889999999999</v>
@@ -6934,24 +6934,24 @@
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C28" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E28">
         <v>4.3285869999999997</v>
@@ -7037,16 +7037,16 @@
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C29" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D29" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E29">
         <v>4.359502</v>
@@ -7132,16 +7132,16 @@
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C30" t="s">
         <v>215</v>
       </c>
       <c r="D30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E30">
         <v>5.7773570000000003</v>
@@ -7227,21 +7227,21 @@
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C32" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E32">
         <v>29310.039062</v>
@@ -7327,16 +7327,16 @@
     </row>
     <row r="33" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B33" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C33" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E33">
         <v>8703.1972659999992</v>
@@ -7422,22 +7422,22 @@
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D34" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="E34" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="F34" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G34">
         <v>2803.3442380000001</v>
@@ -7523,16 +7523,16 @@
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B35" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="C35" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E35">
         <v>5899.8525390000004</v>
@@ -7618,16 +7618,16 @@
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="C36" t="s">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E36">
         <v>2268.0803219999998</v>
@@ -7713,16 +7713,16 @@
     </row>
     <row r="37" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B37" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="C37" t="s">
-        <v>203</v>
+        <v>227</v>
       </c>
       <c r="D37" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E37">
         <v>3631.7719729999999</v>
@@ -7808,16 +7808,16 @@
     </row>
     <row r="38" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B38" t="s">
-        <v>202</v>
+        <v>228</v>
       </c>
       <c r="C38" t="s">
-        <v>201</v>
+        <v>229</v>
       </c>
       <c r="D38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E38">
         <v>38013.234375</v>
@@ -7903,24 +7903,24 @@
     </row>
     <row r="39" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B40" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="D40" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F40">
         <v>341.753174</v>
@@ -8006,19 +8006,19 @@
     </row>
     <row r="41" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
-        <v>198</v>
+        <v>232</v>
       </c>
       <c r="D41" t="s">
-        <v>197</v>
+        <v>233</v>
       </c>
       <c r="E41" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F41">
         <v>278.51181000000003</v>
@@ -8104,19 +8104,19 @@
     </row>
     <row r="42" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>196</v>
+        <v>234</v>
       </c>
       <c r="D42" t="s">
-        <v>195</v>
+        <v>235</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F42">
         <v>63.792053000000003</v>
@@ -8202,19 +8202,19 @@
     </row>
     <row r="43" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B43" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C43" t="s">
-        <v>194</v>
+        <v>236</v>
       </c>
       <c r="D43" t="s">
-        <v>193</v>
+        <v>237</v>
       </c>
       <c r="E43" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F43">
         <v>160.34007299999999</v>
@@ -8300,19 +8300,19 @@
     </row>
     <row r="44" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C44" t="s">
-        <v>192</v>
+        <v>238</v>
       </c>
       <c r="D44" t="s">
-        <v>191</v>
+        <v>239</v>
       </c>
       <c r="E44" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F44">
         <v>12.703077</v>
@@ -8398,21 +8398,21 @@
     </row>
     <row r="45" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B46" t="s">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C46" t="s">
-        <v>189</v>
+        <v>241</v>
       </c>
       <c r="D46" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E46">
         <v>170.75103799999999</v>
@@ -8498,16 +8498,16 @@
     </row>
     <row r="47" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B47" t="s">
-        <v>188</v>
+        <v>242</v>
       </c>
       <c r="C47" t="s">
-        <v>187</v>
+        <v>243</v>
       </c>
       <c r="D47" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E47">
         <v>1.216278</v>
@@ -8593,16 +8593,16 @@
     </row>
     <row r="48" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>244</v>
       </c>
       <c r="C48" t="s">
-        <v>185</v>
+        <v>245</v>
       </c>
       <c r="D48" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E48">
         <v>4.2274219999999998</v>
@@ -8688,21 +8688,21 @@
     </row>
     <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B50" t="s">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="C50" t="s">
-        <v>183</v>
+        <v>247</v>
       </c>
       <c r="D50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E50">
         <v>16819.988281000002</v>
@@ -8788,16 +8788,16 @@
     </row>
     <row r="51" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B51" t="s">
-        <v>182</v>
+        <v>248</v>
       </c>
       <c r="C51" t="s">
-        <v>181</v>
+        <v>249</v>
       </c>
       <c r="D51" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E51">
         <v>1.4477199999999999</v>
@@ -8883,16 +8883,16 @@
     </row>
     <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B52" t="s">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="C52" t="s">
-        <v>179</v>
+        <v>251</v>
       </c>
       <c r="D52" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E52">
         <v>104.64386</v>
@@ -8978,16 +8978,16 @@
     </row>
     <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B53" t="s">
-        <v>178</v>
+        <v>252</v>
       </c>
       <c r="C53" t="s">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="D53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E53">
         <v>15.812405</v>
@@ -9169,16 +9169,16 @@
     </row>
     <row r="3" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E3" s="14">
         <f>'AEO 2025 Table 20'!F6</f>
@@ -9403,9 +9403,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
-    <tabColor theme="8" tint="-0.249977111117893"/>
+    <tabColor rgb="FF1F3864"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9418,10 +9418,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>175</v>
+        <v>254</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>176</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -9439,7 +9439,7 @@
         <v>2025</v>
       </c>
       <c r="B3" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A3,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B2*(1+(('AEO 2026 Table 20'!E6-'AEO 2025 Table 20'!F6)/'AEO 2025 Table 20'!F6))</f>
         <v>21825538331358.785</v>
       </c>
       <c r="F3" s="16"/>
@@ -9449,7 +9449,7 @@
         <v>2026</v>
       </c>
       <c r="B4" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A4,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B3*(1+('AEO 2026 Table 20'!F6/'AEO 2026 Table 20'!E6-1))</f>
         <v>22402540901234.484</v>
       </c>
       <c r="F4" s="16"/>
@@ -9459,7 +9459,7 @@
         <v>2027</v>
       </c>
       <c r="B5" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A5,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B4*(1+('AEO 2026 Table 20'!G6/'AEO 2026 Table 20'!F6-1))</f>
         <v>22823185410025.406</v>
       </c>
       <c r="F5" s="16"/>
@@ -9469,7 +9469,7 @@
         <v>2028</v>
       </c>
       <c r="B6" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A6,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B5*(1+('AEO 2026 Table 20'!H6/'AEO 2026 Table 20'!G6-1))</f>
         <v>23114682186333.645</v>
       </c>
       <c r="F6" s="16"/>
@@ -9479,8 +9479,8 @@
         <v>2029</v>
       </c>
       <c r="B7" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A7,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>23470576225611.391</v>
+        <f>B6*(1+('AEO 2026 Table 20'!I6/'AEO 2026 Table 20'!H6-1))</f>
+        <v>23470576225611.395</v>
       </c>
       <c r="F7" s="16"/>
     </row>
@@ -9489,8 +9489,8 @@
         <v>2030</v>
       </c>
       <c r="B8" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A8,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>23881562591933.387</v>
+        <f>B7*(1+('AEO 2026 Table 20'!J6/'AEO 2026 Table 20'!I6-1))</f>
+        <v>23881562591933.391</v>
       </c>
       <c r="F8" s="16"/>
     </row>
@@ -9499,8 +9499,8 @@
         <v>2031</v>
       </c>
       <c r="B9" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A9,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>24282765360428.699</v>
+        <f>B8*(1+('AEO 2026 Table 20'!K6/'AEO 2026 Table 20'!J6-1))</f>
+        <v>24282765360428.703</v>
       </c>
       <c r="F9" s="16"/>
     </row>
@@ -9509,8 +9509,8 @@
         <v>2032</v>
       </c>
       <c r="B10" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A10,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>24738821126005.746</v>
+        <f>B9*(1+('AEO 2026 Table 20'!L6/'AEO 2026 Table 20'!K6-1))</f>
+        <v>24738821126005.75</v>
       </c>
       <c r="F10" s="16"/>
     </row>
@@ -9519,8 +9519,8 @@
         <v>2033</v>
       </c>
       <c r="B11" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A11,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>25221218682484.555</v>
+        <f>B10*(1+('AEO 2026 Table 20'!M6/'AEO 2026 Table 20'!L6-1))</f>
+        <v>25221218682484.559</v>
       </c>
       <c r="F11" s="16"/>
     </row>
@@ -9529,8 +9529,8 @@
         <v>2034</v>
       </c>
       <c r="B12" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A12,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>25733951374709.305</v>
+        <f>B11*(1+('AEO 2026 Table 20'!N6/'AEO 2026 Table 20'!M6-1))</f>
+        <v>25733951374709.309</v>
       </c>
       <c r="F12" s="16"/>
     </row>
@@ -9539,8 +9539,8 @@
         <v>2035</v>
       </c>
       <c r="B13" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A13,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>26281834762212.441</v>
+        <f>B12*(1+('AEO 2026 Table 20'!O6/'AEO 2026 Table 20'!N6-1))</f>
+        <v>26281834762212.445</v>
       </c>
       <c r="F13" s="16"/>
     </row>
@@ -9549,7 +9549,7 @@
         <v>2036</v>
       </c>
       <c r="B14" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A14,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B13*(1+('AEO 2026 Table 20'!P6/'AEO 2026 Table 20'!O6-1))</f>
         <v>26744394911726.125</v>
       </c>
       <c r="F14" s="16"/>
@@ -9559,7 +9559,7 @@
         <v>2037</v>
       </c>
       <c r="B15" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A15,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B14*(1+('AEO 2026 Table 20'!Q6/'AEO 2026 Table 20'!P6-1))</f>
         <v>27206557464609.492</v>
       </c>
       <c r="F15" s="16"/>
@@ -9569,8 +9569,8 @@
         <v>2038</v>
       </c>
       <c r="B16" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A16,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>27669962991305.672</v>
+        <f>B15*(1+('AEO 2026 Table 20'!R6/'AEO 2026 Table 20'!Q6-1))</f>
+        <v>27669962991305.668</v>
       </c>
       <c r="F16" s="16"/>
     </row>
@@ -9579,8 +9579,8 @@
         <v>2039</v>
       </c>
       <c r="B17" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A17,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>28125300765018.789</v>
+        <f>B16*(1+('AEO 2026 Table 20'!S6/'AEO 2026 Table 20'!R6-1))</f>
+        <v>28125300765018.785</v>
       </c>
       <c r="F17" s="16"/>
     </row>
@@ -9589,7 +9589,7 @@
         <v>2040</v>
       </c>
       <c r="B18" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A18,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B17*(1+('AEO 2026 Table 20'!T6/'AEO 2026 Table 20'!S6-1))</f>
         <v>28584315350240.469</v>
       </c>
       <c r="F18" s="16"/>
@@ -9599,7 +9599,7 @@
         <v>2041</v>
       </c>
       <c r="B19" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A19,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
+        <f>B18*(1+('AEO 2026 Table 20'!U6/'AEO 2026 Table 20'!T6-1))</f>
         <v>29029369634656.645</v>
       </c>
       <c r="F19" s="16"/>
@@ -9609,8 +9609,8 @@
         <v>2042</v>
       </c>
       <c r="B20" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A20,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>29489924427418.73</v>
+        <f>B19*(1+('AEO 2026 Table 20'!V6/'AEO 2026 Table 20'!U6-1))</f>
+        <v>29489924427418.727</v>
       </c>
       <c r="F20" s="16"/>
     </row>
@@ -9619,8 +9619,8 @@
         <v>2043</v>
       </c>
       <c r="B21" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A21,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>29963972438849.711</v>
+        <f>B20*(1+('AEO 2026 Table 20'!W6/'AEO 2026 Table 20'!V6-1))</f>
+        <v>29963972438849.707</v>
       </c>
       <c r="F21" s="16"/>
     </row>
@@ -9629,8 +9629,8 @@
         <v>2044</v>
       </c>
       <c r="B22" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A22,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>30442799339569.688</v>
+        <f>B21*(1+('AEO 2026 Table 20'!X6/'AEO 2026 Table 20'!W6-1))</f>
+        <v>30442799339569.684</v>
       </c>
       <c r="F22" s="16"/>
     </row>
@@ -9639,8 +9639,8 @@
         <v>2045</v>
       </c>
       <c r="B23" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A23,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>30925000027200.043</v>
+        <f>B22*(1+('AEO 2026 Table 20'!Y6/'AEO 2026 Table 20'!X6-1))</f>
+        <v>30925000027200.035</v>
       </c>
       <c r="F23" s="16"/>
     </row>
@@ -9649,8 +9649,8 @@
         <v>2046</v>
       </c>
       <c r="B24" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A24,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>31395153128705.172</v>
+        <f>B23*(1+('AEO 2026 Table 20'!Z6/'AEO 2026 Table 20'!Y6-1))</f>
+        <v>31395153128705.168</v>
       </c>
       <c r="F24" s="16"/>
     </row>
@@ -9659,8 +9659,8 @@
         <v>2047</v>
       </c>
       <c r="B25" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A25,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>31846296829792.25</v>
+        <f>B24*(1+('AEO 2026 Table 20'!AA6/'AEO 2026 Table 20'!Z6-1))</f>
+        <v>31846296829792.242</v>
       </c>
       <c r="F25" s="16"/>
     </row>
@@ -9669,8 +9669,8 @@
         <v>2048</v>
       </c>
       <c r="B26" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A26,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>32295491145955.598</v>
+        <f>B25*(1+('AEO 2026 Table 20'!AB6/'AEO 2026 Table 20'!AA6-1))</f>
+        <v>32295491145955.59</v>
       </c>
       <c r="F26" s="16"/>
     </row>
@@ -9679,8 +9679,8 @@
         <v>2049</v>
       </c>
       <c r="B27" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A27,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>32734311257746.891</v>
+        <f>B26*(1+('AEO 2026 Table 20'!AC6/'AEO 2026 Table 20'!AB6-1))</f>
+        <v>32734311257746.883</v>
       </c>
       <c r="F27" s="16"/>
     </row>
@@ -9689,8 +9689,8 @@
         <v>2050</v>
       </c>
       <c r="B28" s="19">
-        <f>$B$2*INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A28,calcs!$E$2:$AF$2,0))/INDEX(calcs!$E$3:$AF$3,MATCH(BGDP!A$2,calcs!$E$2:$AF$2,0))</f>
-        <v>33186777066968.887</v>
+        <f>B27*(1+('AEO 2026 Table 20'!AD6/'AEO 2026 Table 20'!AC6-1))</f>
+        <v>33186777066968.883</v>
       </c>
       <c r="F28" s="16"/>
     </row>

</xml_diff>